<commit_message>
deploy: main → 05c809bec3570b713cac4ddcf8254383a752aafc
</commit_message>
<xml_diff>
--- a/StructureDefinition-inera-ehds-document-reference.xlsx
+++ b/StructureDefinition-inera-ehds-document-reference.xlsx
@@ -10,13 +10,13 @@
     <sheet name="Elements" r:id="rId4" sheetId="2"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="true">Elements!$A$1:$AQ$64</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="true">Elements!$A$1:$AQ$65</definedName>
   </definedNames>
 </workbook>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="2534" uniqueCount="518">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="2571" uniqueCount="525">
   <si>
     <t>Property</t>
   </si>
@@ -60,7 +60,7 @@
     <t>Date</t>
   </si>
   <si>
-    <t>2026-09-30T10:52:57+00:00</t>
+    <t>2026-10-01T18:35:17+00:00</t>
   </si>
   <si>
     <t>Publisher</t>
@@ -624,10 +624,33 @@
     <t>DocumentReference.extension</t>
   </si>
   <si>
-    <t>May be used to represent additional information that is not part of the basic definition of the resource. To make the use of extensions safe and manageable, there is a strict set of governance  applied to the definition and use of extensions. Though any implementer can define an extension, there is a set of requirements that SHALL be met as part of the definition of the extension.</t>
+    <t>Extension</t>
+  </si>
+  <si>
+    <t>An Extension</t>
   </si>
   <si>
     <t>DomainResource.extension</t>
+  </si>
+  <si>
+    <t>DocumentReference.extension:ext-signature-time</t>
+  </si>
+  <si>
+    <t>ext-signature-time</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Extension {https://fhir.inera.se/ig/ehds-tk/StructureDefinition/ext-signature-time}
+</t>
+  </si>
+  <si>
+    <t>Signeringstidpunkt (careDocumentation.header.signature.timestamp) – utelämnas om signature.timestamp saknas (DOC-003)</t>
+  </si>
+  <si>
+    <t>Tidpunkt då journalanteckningen signerades (careDocumentation.header.signature.timestamp, JoL-header v2.2). Anges endast när signature.timestamp finns i källan; ingen ersättningstidpunkt sätts annars. Se DOC-003.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">ele-1
+</t>
   </si>
   <si>
     <t>DocumentReference.modifierExtension</t>
@@ -1206,7 +1229,7 @@
     <t>DocumentReference.content.attachment.contentType</t>
   </si>
   <si>
-    <t>Mimetyp (careDocumentation.body.multimediaEntry.mediaType)</t>
+    <t>Mimetyp (careDocumentation.body.multimediaEntry.mediaType); för clinicalDocumentNoteText text/plain; charset=utf-8 (fritext) eller text/html; charset=utf-8 (DocBook → XHTML, DOC-004)</t>
   </si>
   <si>
     <t>Identifies the type of the data in the attachment and allows a method to be chosen to interpret or render the data. Includes mime type parameters such as charset where appropriate.</t>
@@ -1261,7 +1284,7 @@
 </t>
   </si>
   <si>
-    <t>Anteckningstext/binärinnehåll (careDocumentation.body.clinicalDocumentNoteText / multimediaEntry.value)</t>
+    <t>Anteckningstext/binärinnehåll (careDocumentation.body.clinicalDocumentNoteText / multimediaEntry.value) – för clinicalDocumentNoteText: fritext base64-kodas som text/plain; DocBook-XML transformeras till XHTML och base64-kodas som text/html (DOC-004)</t>
   </si>
   <si>
     <t>The actual data of the attachment - a sequence of bytes, base64 encoded.</t>
@@ -1940,12 +1963,12 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <dimension ref="A1:AQ64"/>
+  <dimension ref="A1:AQ65"/>
   <sheetFormatPr defaultRowHeight="15.0"/>
   <cols>
     <col min="1" max="1" width="43.578125" customWidth="true" bestFit="true"/>
     <col min="2" max="2" width="43.578125" customWidth="true" bestFit="true"/>
-    <col min="3" max="3" width="10.8515625" customWidth="true" bestFit="true" hidden="true"/>
+    <col min="3" max="3" width="15.53125" customWidth="true" bestFit="true" hidden="true"/>
     <col min="4" max="4" width="34.21875" customWidth="true" bestFit="true" hidden="true"/>
     <col min="5" max="5" width="5.80859375" customWidth="true" bestFit="true"/>
     <col min="6" max="6" width="4.23828125" customWidth="true" bestFit="true"/>
@@ -3968,7 +3991,7 @@
       </c>
       <c r="C17" s="2"/>
       <c r="D17" t="s" s="2">
-        <v>113</v>
+        <v>80</v>
       </c>
       <c r="E17" s="2"/>
       <c r="F17" t="s" s="2">
@@ -3990,14 +4013,12 @@
         <v>114</v>
       </c>
       <c r="L17" t="s" s="2">
-        <v>115</v>
+        <v>194</v>
       </c>
       <c r="M17" t="s" s="2">
-        <v>194</v>
-      </c>
-      <c r="N17" t="s" s="2">
-        <v>117</v>
-      </c>
+        <v>195</v>
+      </c>
+      <c r="N17" s="2"/>
       <c r="O17" s="2"/>
       <c r="P17" t="s" s="2">
         <v>80</v>
@@ -4034,19 +4055,17 @@
         <v>80</v>
       </c>
       <c r="AB17" t="s" s="2">
-        <v>80</v>
-      </c>
-      <c r="AC17" t="s" s="2">
-        <v>80</v>
-      </c>
+        <v>118</v>
+      </c>
+      <c r="AC17" s="2"/>
       <c r="AD17" t="s" s="2">
         <v>80</v>
       </c>
       <c r="AE17" t="s" s="2">
-        <v>80</v>
+        <v>120</v>
       </c>
       <c r="AF17" t="s" s="2">
-        <v>195</v>
+        <v>196</v>
       </c>
       <c r="AG17" t="s" s="2">
         <v>81</v>
@@ -4067,7 +4086,7 @@
         <v>80</v>
       </c>
       <c r="AM17" t="s" s="2">
-        <v>192</v>
+        <v>80</v>
       </c>
       <c r="AN17" t="s" s="2">
         <v>80</v>
@@ -4082,48 +4101,46 @@
         <v>80</v>
       </c>
     </row>
-    <row r="18" hidden="true">
+    <row r="18">
       <c r="A18" t="s" s="2">
-        <v>196</v>
+        <v>197</v>
       </c>
       <c r="B18" t="s" s="2">
-        <v>196</v>
-      </c>
-      <c r="C18" s="2"/>
+        <v>193</v>
+      </c>
+      <c r="C18" t="s" s="2">
+        <v>198</v>
+      </c>
       <c r="D18" t="s" s="2">
-        <v>113</v>
+        <v>80</v>
       </c>
       <c r="E18" s="2"/>
       <c r="F18" t="s" s="2">
         <v>81</v>
       </c>
       <c r="G18" t="s" s="2">
-        <v>82</v>
+        <v>93</v>
       </c>
       <c r="H18" t="s" s="2">
-        <v>80</v>
+        <v>94</v>
       </c>
       <c r="I18" t="s" s="2">
-        <v>94</v>
+        <v>80</v>
       </c>
       <c r="J18" t="s" s="2">
         <v>80</v>
       </c>
       <c r="K18" t="s" s="2">
-        <v>114</v>
+        <v>199</v>
       </c>
       <c r="L18" t="s" s="2">
-        <v>197</v>
+        <v>200</v>
       </c>
       <c r="M18" t="s" s="2">
-        <v>198</v>
-      </c>
-      <c r="N18" t="s" s="2">
-        <v>117</v>
-      </c>
-      <c r="O18" t="s" s="2">
-        <v>199</v>
-      </c>
+        <v>201</v>
+      </c>
+      <c r="N18" s="2"/>
+      <c r="O18" s="2"/>
       <c r="P18" t="s" s="2">
         <v>80</v>
       </c>
@@ -4171,7 +4188,7 @@
         <v>80</v>
       </c>
       <c r="AF18" t="s" s="2">
-        <v>200</v>
+        <v>196</v>
       </c>
       <c r="AG18" t="s" s="2">
         <v>81</v>
@@ -4180,7 +4197,7 @@
         <v>82</v>
       </c>
       <c r="AI18" t="s" s="2">
-        <v>80</v>
+        <v>202</v>
       </c>
       <c r="AJ18" t="s" s="2">
         <v>122</v>
@@ -4192,7 +4209,7 @@
         <v>80</v>
       </c>
       <c r="AM18" t="s" s="2">
-        <v>192</v>
+        <v>80</v>
       </c>
       <c r="AN18" t="s" s="2">
         <v>80</v>
@@ -4209,42 +4226,42 @@
     </row>
     <row r="19" hidden="true">
       <c r="A19" t="s" s="2">
-        <v>201</v>
+        <v>203</v>
       </c>
       <c r="B19" t="s" s="2">
-        <v>201</v>
+        <v>203</v>
       </c>
       <c r="C19" s="2"/>
       <c r="D19" t="s" s="2">
-        <v>80</v>
+        <v>113</v>
       </c>
       <c r="E19" s="2"/>
       <c r="F19" t="s" s="2">
         <v>81</v>
       </c>
       <c r="G19" t="s" s="2">
-        <v>93</v>
+        <v>82</v>
       </c>
       <c r="H19" t="s" s="2">
         <v>80</v>
       </c>
       <c r="I19" t="s" s="2">
-        <v>80</v>
+        <v>94</v>
       </c>
       <c r="J19" t="s" s="2">
-        <v>94</v>
+        <v>80</v>
       </c>
       <c r="K19" t="s" s="2">
-        <v>202</v>
+        <v>114</v>
       </c>
       <c r="L19" t="s" s="2">
-        <v>203</v>
+        <v>204</v>
       </c>
       <c r="M19" t="s" s="2">
-        <v>204</v>
+        <v>205</v>
       </c>
       <c r="N19" t="s" s="2">
-        <v>205</v>
+        <v>117</v>
       </c>
       <c r="O19" t="s" s="2">
         <v>206</v>
@@ -4296,48 +4313,48 @@
         <v>80</v>
       </c>
       <c r="AF19" t="s" s="2">
-        <v>201</v>
+        <v>207</v>
       </c>
       <c r="AG19" t="s" s="2">
         <v>81</v>
       </c>
       <c r="AH19" t="s" s="2">
-        <v>93</v>
+        <v>82</v>
       </c>
       <c r="AI19" t="s" s="2">
         <v>80</v>
       </c>
       <c r="AJ19" t="s" s="2">
-        <v>105</v>
+        <v>122</v>
       </c>
       <c r="AK19" t="s" s="2">
-        <v>207</v>
+        <v>80</v>
       </c>
       <c r="AL19" t="s" s="2">
-        <v>208</v>
+        <v>80</v>
       </c>
       <c r="AM19" t="s" s="2">
-        <v>209</v>
+        <v>192</v>
       </c>
       <c r="AN19" t="s" s="2">
-        <v>210</v>
+        <v>80</v>
       </c>
       <c r="AO19" t="s" s="2">
-        <v>211</v>
+        <v>80</v>
       </c>
       <c r="AP19" t="s" s="2">
-        <v>212</v>
+        <v>80</v>
       </c>
       <c r="AQ19" t="s" s="2">
-        <v>213</v>
+        <v>80</v>
       </c>
     </row>
     <row r="20" hidden="true">
       <c r="A20" t="s" s="2">
-        <v>214</v>
+        <v>208</v>
       </c>
       <c r="B20" t="s" s="2">
-        <v>214</v>
+        <v>208</v>
       </c>
       <c r="C20" s="2"/>
       <c r="D20" t="s" s="2">
@@ -4348,7 +4365,7 @@
         <v>81</v>
       </c>
       <c r="G20" t="s" s="2">
-        <v>82</v>
+        <v>93</v>
       </c>
       <c r="H20" t="s" s="2">
         <v>80</v>
@@ -4360,16 +4377,20 @@
         <v>94</v>
       </c>
       <c r="K20" t="s" s="2">
-        <v>202</v>
+        <v>209</v>
       </c>
       <c r="L20" t="s" s="2">
-        <v>215</v>
+        <v>210</v>
       </c>
       <c r="M20" t="s" s="2">
-        <v>216</v>
-      </c>
-      <c r="N20" s="2"/>
-      <c r="O20" s="2"/>
+        <v>211</v>
+      </c>
+      <c r="N20" t="s" s="2">
+        <v>212</v>
+      </c>
+      <c r="O20" t="s" s="2">
+        <v>213</v>
+      </c>
       <c r="P20" t="s" s="2">
         <v>80</v>
       </c>
@@ -4417,13 +4438,13 @@
         <v>80</v>
       </c>
       <c r="AF20" t="s" s="2">
-        <v>214</v>
+        <v>208</v>
       </c>
       <c r="AG20" t="s" s="2">
         <v>81</v>
       </c>
       <c r="AH20" t="s" s="2">
-        <v>82</v>
+        <v>93</v>
       </c>
       <c r="AI20" t="s" s="2">
         <v>80</v>
@@ -4432,33 +4453,33 @@
         <v>105</v>
       </c>
       <c r="AK20" t="s" s="2">
-        <v>207</v>
+        <v>214</v>
       </c>
       <c r="AL20" t="s" s="2">
-        <v>80</v>
+        <v>215</v>
       </c>
       <c r="AM20" t="s" s="2">
+        <v>216</v>
+      </c>
+      <c r="AN20" t="s" s="2">
         <v>217</v>
       </c>
-      <c r="AN20" t="s" s="2">
-        <v>80</v>
-      </c>
       <c r="AO20" t="s" s="2">
-        <v>211</v>
+        <v>218</v>
       </c>
       <c r="AP20" t="s" s="2">
-        <v>218</v>
+        <v>219</v>
       </c>
       <c r="AQ20" t="s" s="2">
-        <v>219</v>
+        <v>220</v>
       </c>
     </row>
-    <row r="21">
+    <row r="21" hidden="true">
       <c r="A21" t="s" s="2">
-        <v>220</v>
+        <v>221</v>
       </c>
       <c r="B21" t="s" s="2">
-        <v>220</v>
+        <v>221</v>
       </c>
       <c r="C21" s="2"/>
       <c r="D21" t="s" s="2">
@@ -4466,32 +4487,30 @@
       </c>
       <c r="E21" s="2"/>
       <c r="F21" t="s" s="2">
-        <v>93</v>
+        <v>81</v>
       </c>
       <c r="G21" t="s" s="2">
-        <v>93</v>
+        <v>82</v>
       </c>
       <c r="H21" t="s" s="2">
-        <v>94</v>
+        <v>80</v>
       </c>
       <c r="I21" t="s" s="2">
-        <v>94</v>
+        <v>80</v>
       </c>
       <c r="J21" t="s" s="2">
         <v>94</v>
       </c>
       <c r="K21" t="s" s="2">
-        <v>169</v>
+        <v>209</v>
       </c>
       <c r="L21" t="s" s="2">
-        <v>221</v>
+        <v>222</v>
       </c>
       <c r="M21" t="s" s="2">
-        <v>222</v>
-      </c>
-      <c r="N21" t="s" s="2">
         <v>223</v>
       </c>
+      <c r="N21" s="2"/>
       <c r="O21" s="2"/>
       <c r="P21" t="s" s="2">
         <v>80</v>
@@ -4516,13 +4535,13 @@
         <v>80</v>
       </c>
       <c r="X21" t="s" s="2">
-        <v>224</v>
+        <v>80</v>
       </c>
       <c r="Y21" t="s" s="2">
-        <v>225</v>
+        <v>80</v>
       </c>
       <c r="Z21" t="s" s="2">
-        <v>226</v>
+        <v>80</v>
       </c>
       <c r="AA21" t="s" s="2">
         <v>80</v>
@@ -4540,13 +4559,13 @@
         <v>80</v>
       </c>
       <c r="AF21" t="s" s="2">
-        <v>220</v>
+        <v>221</v>
       </c>
       <c r="AG21" t="s" s="2">
-        <v>93</v>
+        <v>81</v>
       </c>
       <c r="AH21" t="s" s="2">
-        <v>93</v>
+        <v>82</v>
       </c>
       <c r="AI21" t="s" s="2">
         <v>80</v>
@@ -4555,33 +4574,33 @@
         <v>105</v>
       </c>
       <c r="AK21" t="s" s="2">
+        <v>214</v>
+      </c>
+      <c r="AL21" t="s" s="2">
+        <v>80</v>
+      </c>
+      <c r="AM21" t="s" s="2">
+        <v>224</v>
+      </c>
+      <c r="AN21" t="s" s="2">
+        <v>80</v>
+      </c>
+      <c r="AO21" t="s" s="2">
+        <v>218</v>
+      </c>
+      <c r="AP21" t="s" s="2">
+        <v>225</v>
+      </c>
+      <c r="AQ21" t="s" s="2">
+        <v>226</v>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" t="s" s="2">
         <v>227</v>
       </c>
-      <c r="AL21" t="s" s="2">
-        <v>80</v>
-      </c>
-      <c r="AM21" t="s" s="2">
-        <v>228</v>
-      </c>
-      <c r="AN21" t="s" s="2">
-        <v>80</v>
-      </c>
-      <c r="AO21" t="s" s="2">
-        <v>229</v>
-      </c>
-      <c r="AP21" t="s" s="2">
-        <v>230</v>
-      </c>
-      <c r="AQ21" t="s" s="2">
-        <v>231</v>
-      </c>
-    </row>
-    <row r="22" hidden="true">
-      <c r="A22" t="s" s="2">
-        <v>232</v>
-      </c>
       <c r="B22" t="s" s="2">
-        <v>232</v>
+        <v>227</v>
       </c>
       <c r="C22" s="2"/>
       <c r="D22" t="s" s="2">
@@ -4589,16 +4608,16 @@
       </c>
       <c r="E22" s="2"/>
       <c r="F22" t="s" s="2">
-        <v>81</v>
+        <v>93</v>
       </c>
       <c r="G22" t="s" s="2">
         <v>93</v>
       </c>
       <c r="H22" t="s" s="2">
-        <v>80</v>
+        <v>94</v>
       </c>
       <c r="I22" t="s" s="2">
-        <v>80</v>
+        <v>94</v>
       </c>
       <c r="J22" t="s" s="2">
         <v>94</v>
@@ -4607,13 +4626,13 @@
         <v>169</v>
       </c>
       <c r="L22" t="s" s="2">
-        <v>233</v>
+        <v>228</v>
       </c>
       <c r="M22" t="s" s="2">
-        <v>234</v>
+        <v>229</v>
       </c>
       <c r="N22" t="s" s="2">
-        <v>235</v>
+        <v>230</v>
       </c>
       <c r="O22" s="2"/>
       <c r="P22" t="s" s="2">
@@ -4639,13 +4658,13 @@
         <v>80</v>
       </c>
       <c r="X22" t="s" s="2">
-        <v>224</v>
+        <v>231</v>
       </c>
       <c r="Y22" t="s" s="2">
-        <v>236</v>
+        <v>232</v>
       </c>
       <c r="Z22" t="s" s="2">
-        <v>237</v>
+        <v>233</v>
       </c>
       <c r="AA22" t="s" s="2">
         <v>80</v>
@@ -4663,10 +4682,10 @@
         <v>80</v>
       </c>
       <c r="AF22" t="s" s="2">
-        <v>232</v>
+        <v>227</v>
       </c>
       <c r="AG22" t="s" s="2">
-        <v>81</v>
+        <v>93</v>
       </c>
       <c r="AH22" t="s" s="2">
         <v>93</v>
@@ -4678,33 +4697,33 @@
         <v>105</v>
       </c>
       <c r="AK22" t="s" s="2">
-        <v>80</v>
+        <v>234</v>
       </c>
       <c r="AL22" t="s" s="2">
+        <v>80</v>
+      </c>
+      <c r="AM22" t="s" s="2">
+        <v>235</v>
+      </c>
+      <c r="AN22" t="s" s="2">
+        <v>80</v>
+      </c>
+      <c r="AO22" t="s" s="2">
+        <v>236</v>
+      </c>
+      <c r="AP22" t="s" s="2">
+        <v>237</v>
+      </c>
+      <c r="AQ22" t="s" s="2">
         <v>238</v>
       </c>
-      <c r="AM22" t="s" s="2">
+    </row>
+    <row r="23" hidden="true">
+      <c r="A23" t="s" s="2">
         <v>239</v>
       </c>
-      <c r="AN22" t="s" s="2">
-        <v>80</v>
-      </c>
-      <c r="AO22" t="s" s="2">
-        <v>229</v>
-      </c>
-      <c r="AP22" t="s" s="2">
-        <v>240</v>
-      </c>
-      <c r="AQ22" t="s" s="2">
-        <v>80</v>
-      </c>
-    </row>
-    <row r="23">
-      <c r="A23" t="s" s="2">
-        <v>241</v>
-      </c>
       <c r="B23" t="s" s="2">
-        <v>241</v>
+        <v>239</v>
       </c>
       <c r="C23" s="2"/>
       <c r="D23" t="s" s="2">
@@ -4718,7 +4737,7 @@
         <v>93</v>
       </c>
       <c r="H23" t="s" s="2">
-        <v>94</v>
+        <v>80</v>
       </c>
       <c r="I23" t="s" s="2">
         <v>80</v>
@@ -4727,16 +4746,16 @@
         <v>94</v>
       </c>
       <c r="K23" t="s" s="2">
+        <v>169</v>
+      </c>
+      <c r="L23" t="s" s="2">
+        <v>240</v>
+      </c>
+      <c r="M23" t="s" s="2">
+        <v>241</v>
+      </c>
+      <c r="N23" t="s" s="2">
         <v>242</v>
-      </c>
-      <c r="L23" t="s" s="2">
-        <v>243</v>
-      </c>
-      <c r="M23" t="s" s="2">
-        <v>244</v>
-      </c>
-      <c r="N23" t="s" s="2">
-        <v>245</v>
       </c>
       <c r="O23" s="2"/>
       <c r="P23" t="s" s="2">
@@ -4762,13 +4781,13 @@
         <v>80</v>
       </c>
       <c r="X23" t="s" s="2">
-        <v>173</v>
+        <v>231</v>
       </c>
       <c r="Y23" t="s" s="2">
-        <v>246</v>
+        <v>243</v>
       </c>
       <c r="Z23" t="s" s="2">
-        <v>247</v>
+        <v>244</v>
       </c>
       <c r="AA23" t="s" s="2">
         <v>80</v>
@@ -4786,7 +4805,7 @@
         <v>80</v>
       </c>
       <c r="AF23" t="s" s="2">
-        <v>241</v>
+        <v>239</v>
       </c>
       <c r="AG23" t="s" s="2">
         <v>81</v>
@@ -4801,44 +4820,44 @@
         <v>105</v>
       </c>
       <c r="AK23" t="s" s="2">
-        <v>248</v>
+        <v>80</v>
       </c>
       <c r="AL23" t="s" s="2">
-        <v>249</v>
+        <v>245</v>
       </c>
       <c r="AM23" t="s" s="2">
-        <v>250</v>
+        <v>246</v>
       </c>
       <c r="AN23" t="s" s="2">
-        <v>251</v>
+        <v>80</v>
       </c>
       <c r="AO23" t="s" s="2">
-        <v>252</v>
+        <v>236</v>
       </c>
       <c r="AP23" t="s" s="2">
-        <v>253</v>
+        <v>247</v>
       </c>
       <c r="AQ23" t="s" s="2">
-        <v>254</v>
+        <v>80</v>
       </c>
     </row>
     <row r="24">
       <c r="A24" t="s" s="2">
-        <v>255</v>
+        <v>248</v>
       </c>
       <c r="B24" t="s" s="2">
-        <v>255</v>
+        <v>248</v>
       </c>
       <c r="C24" s="2"/>
       <c r="D24" t="s" s="2">
-        <v>256</v>
+        <v>80</v>
       </c>
       <c r="E24" s="2"/>
       <c r="F24" t="s" s="2">
         <v>81</v>
       </c>
       <c r="G24" t="s" s="2">
-        <v>82</v>
+        <v>93</v>
       </c>
       <c r="H24" t="s" s="2">
         <v>94</v>
@@ -4850,16 +4869,16 @@
         <v>94</v>
       </c>
       <c r="K24" t="s" s="2">
-        <v>242</v>
+        <v>249</v>
       </c>
       <c r="L24" t="s" s="2">
-        <v>257</v>
+        <v>250</v>
       </c>
       <c r="M24" t="s" s="2">
-        <v>258</v>
+        <v>251</v>
       </c>
       <c r="N24" t="s" s="2">
-        <v>259</v>
+        <v>252</v>
       </c>
       <c r="O24" s="2"/>
       <c r="P24" t="s" s="2">
@@ -4885,13 +4904,13 @@
         <v>80</v>
       </c>
       <c r="X24" t="s" s="2">
-        <v>159</v>
+        <v>173</v>
       </c>
       <c r="Y24" t="s" s="2">
-        <v>260</v>
+        <v>253</v>
       </c>
       <c r="Z24" t="s" s="2">
-        <v>261</v>
+        <v>254</v>
       </c>
       <c r="AA24" t="s" s="2">
         <v>80</v>
@@ -4909,13 +4928,13 @@
         <v>80</v>
       </c>
       <c r="AF24" t="s" s="2">
-        <v>255</v>
+        <v>248</v>
       </c>
       <c r="AG24" t="s" s="2">
         <v>81</v>
       </c>
       <c r="AH24" t="s" s="2">
-        <v>82</v>
+        <v>93</v>
       </c>
       <c r="AI24" t="s" s="2">
         <v>80</v>
@@ -4924,44 +4943,44 @@
         <v>105</v>
       </c>
       <c r="AK24" t="s" s="2">
-        <v>80</v>
+        <v>255</v>
       </c>
       <c r="AL24" t="s" s="2">
-        <v>262</v>
+        <v>256</v>
       </c>
       <c r="AM24" t="s" s="2">
-        <v>263</v>
+        <v>257</v>
       </c>
       <c r="AN24" t="s" s="2">
-        <v>264</v>
+        <v>258</v>
       </c>
       <c r="AO24" t="s" s="2">
-        <v>252</v>
+        <v>259</v>
       </c>
       <c r="AP24" t="s" s="2">
-        <v>80</v>
+        <v>260</v>
       </c>
       <c r="AQ24" t="s" s="2">
-        <v>265</v>
+        <v>261</v>
       </c>
     </row>
     <row r="25">
       <c r="A25" t="s" s="2">
-        <v>266</v>
+        <v>262</v>
       </c>
       <c r="B25" t="s" s="2">
-        <v>266</v>
+        <v>262</v>
       </c>
       <c r="C25" s="2"/>
       <c r="D25" t="s" s="2">
-        <v>80</v>
+        <v>263</v>
       </c>
       <c r="E25" s="2"/>
       <c r="F25" t="s" s="2">
         <v>81</v>
       </c>
       <c r="G25" t="s" s="2">
-        <v>93</v>
+        <v>82</v>
       </c>
       <c r="H25" t="s" s="2">
         <v>94</v>
@@ -4973,15 +4992,17 @@
         <v>94</v>
       </c>
       <c r="K25" t="s" s="2">
-        <v>267</v>
+        <v>249</v>
       </c>
       <c r="L25" t="s" s="2">
-        <v>268</v>
+        <v>264</v>
       </c>
       <c r="M25" t="s" s="2">
-        <v>269</v>
-      </c>
-      <c r="N25" s="2"/>
+        <v>265</v>
+      </c>
+      <c r="N25" t="s" s="2">
+        <v>266</v>
+      </c>
       <c r="O25" s="2"/>
       <c r="P25" t="s" s="2">
         <v>80</v>
@@ -5006,13 +5027,13 @@
         <v>80</v>
       </c>
       <c r="X25" t="s" s="2">
-        <v>80</v>
+        <v>159</v>
       </c>
       <c r="Y25" t="s" s="2">
-        <v>80</v>
+        <v>267</v>
       </c>
       <c r="Z25" t="s" s="2">
-        <v>80</v>
+        <v>268</v>
       </c>
       <c r="AA25" t="s" s="2">
         <v>80</v>
@@ -5030,13 +5051,13 @@
         <v>80</v>
       </c>
       <c r="AF25" t="s" s="2">
-        <v>266</v>
+        <v>262</v>
       </c>
       <c r="AG25" t="s" s="2">
         <v>81</v>
       </c>
       <c r="AH25" t="s" s="2">
-        <v>93</v>
+        <v>82</v>
       </c>
       <c r="AI25" t="s" s="2">
         <v>80</v>
@@ -5045,37 +5066,37 @@
         <v>105</v>
       </c>
       <c r="AK25" t="s" s="2">
+        <v>80</v>
+      </c>
+      <c r="AL25" t="s" s="2">
+        <v>269</v>
+      </c>
+      <c r="AM25" t="s" s="2">
         <v>270</v>
       </c>
-      <c r="AL25" t="s" s="2">
+      <c r="AN25" t="s" s="2">
         <v>271</v>
       </c>
-      <c r="AM25" t="s" s="2">
+      <c r="AO25" t="s" s="2">
+        <v>259</v>
+      </c>
+      <c r="AP25" t="s" s="2">
+        <v>80</v>
+      </c>
+      <c r="AQ25" t="s" s="2">
         <v>272</v>
-      </c>
-      <c r="AN25" t="s" s="2">
-        <v>273</v>
-      </c>
-      <c r="AO25" t="s" s="2">
-        <v>274</v>
-      </c>
-      <c r="AP25" t="s" s="2">
-        <v>275</v>
-      </c>
-      <c r="AQ25" t="s" s="2">
-        <v>276</v>
       </c>
     </row>
     <row r="26">
       <c r="A26" t="s" s="2">
-        <v>277</v>
+        <v>273</v>
       </c>
       <c r="B26" t="s" s="2">
-        <v>277</v>
+        <v>273</v>
       </c>
       <c r="C26" s="2"/>
       <c r="D26" t="s" s="2">
-        <v>278</v>
+        <v>80</v>
       </c>
       <c r="E26" s="2"/>
       <c r="F26" t="s" s="2">
@@ -5094,17 +5115,15 @@
         <v>94</v>
       </c>
       <c r="K26" t="s" s="2">
-        <v>129</v>
+        <v>274</v>
       </c>
       <c r="L26" t="s" s="2">
-        <v>279</v>
+        <v>275</v>
       </c>
       <c r="M26" t="s" s="2">
-        <v>280</v>
-      </c>
-      <c r="N26" t="s" s="2">
-        <v>281</v>
-      </c>
+        <v>276</v>
+      </c>
+      <c r="N26" s="2"/>
       <c r="O26" s="2"/>
       <c r="P26" t="s" s="2">
         <v>80</v>
@@ -5153,7 +5172,7 @@
         <v>80</v>
       </c>
       <c r="AF26" t="s" s="2">
-        <v>277</v>
+        <v>273</v>
       </c>
       <c r="AG26" t="s" s="2">
         <v>81</v>
@@ -5168,44 +5187,44 @@
         <v>105</v>
       </c>
       <c r="AK26" t="s" s="2">
+        <v>277</v>
+      </c>
+      <c r="AL26" t="s" s="2">
+        <v>278</v>
+      </c>
+      <c r="AM26" t="s" s="2">
+        <v>279</v>
+      </c>
+      <c r="AN26" t="s" s="2">
+        <v>280</v>
+      </c>
+      <c r="AO26" t="s" s="2">
+        <v>281</v>
+      </c>
+      <c r="AP26" t="s" s="2">
         <v>282</v>
       </c>
-      <c r="AL26" t="s" s="2">
+      <c r="AQ26" t="s" s="2">
         <v>283</v>
-      </c>
-      <c r="AM26" t="s" s="2">
-        <v>284</v>
-      </c>
-      <c r="AN26" t="s" s="2">
-        <v>80</v>
-      </c>
-      <c r="AO26" t="s" s="2">
-        <v>285</v>
-      </c>
-      <c r="AP26" t="s" s="2">
-        <v>80</v>
-      </c>
-      <c r="AQ26" t="s" s="2">
-        <v>80</v>
       </c>
     </row>
     <row r="27">
       <c r="A27" t="s" s="2">
-        <v>286</v>
+        <v>284</v>
       </c>
       <c r="B27" t="s" s="2">
-        <v>286</v>
+        <v>284</v>
       </c>
       <c r="C27" s="2"/>
       <c r="D27" t="s" s="2">
-        <v>80</v>
+        <v>285</v>
       </c>
       <c r="E27" s="2"/>
       <c r="F27" t="s" s="2">
         <v>81</v>
       </c>
       <c r="G27" t="s" s="2">
-        <v>82</v>
+        <v>93</v>
       </c>
       <c r="H27" t="s" s="2">
         <v>94</v>
@@ -5217,16 +5236,16 @@
         <v>94</v>
       </c>
       <c r="K27" t="s" s="2">
+        <v>129</v>
+      </c>
+      <c r="L27" t="s" s="2">
+        <v>286</v>
+      </c>
+      <c r="M27" t="s" s="2">
         <v>287</v>
       </c>
-      <c r="L27" t="s" s="2">
+      <c r="N27" t="s" s="2">
         <v>288</v>
-      </c>
-      <c r="M27" t="s" s="2">
-        <v>289</v>
-      </c>
-      <c r="N27" t="s" s="2">
-        <v>290</v>
       </c>
       <c r="O27" s="2"/>
       <c r="P27" t="s" s="2">
@@ -5276,13 +5295,13 @@
         <v>80</v>
       </c>
       <c r="AF27" t="s" s="2">
-        <v>286</v>
+        <v>284</v>
       </c>
       <c r="AG27" t="s" s="2">
         <v>81</v>
       </c>
       <c r="AH27" t="s" s="2">
-        <v>82</v>
+        <v>93</v>
       </c>
       <c r="AI27" t="s" s="2">
         <v>80</v>
@@ -5291,33 +5310,33 @@
         <v>105</v>
       </c>
       <c r="AK27" t="s" s="2">
+        <v>289</v>
+      </c>
+      <c r="AL27" t="s" s="2">
+        <v>290</v>
+      </c>
+      <c r="AM27" t="s" s="2">
         <v>291</v>
       </c>
-      <c r="AL27" t="s" s="2">
+      <c r="AN27" t="s" s="2">
+        <v>80</v>
+      </c>
+      <c r="AO27" t="s" s="2">
         <v>292</v>
       </c>
-      <c r="AM27" t="s" s="2">
-        <v>293</v>
-      </c>
-      <c r="AN27" t="s" s="2">
-        <v>294</v>
-      </c>
-      <c r="AO27" t="s" s="2">
-        <v>80</v>
-      </c>
       <c r="AP27" t="s" s="2">
-        <v>295</v>
+        <v>80</v>
       </c>
       <c r="AQ27" t="s" s="2">
-        <v>296</v>
+        <v>80</v>
       </c>
     </row>
     <row r="28">
       <c r="A28" t="s" s="2">
-        <v>297</v>
+        <v>293</v>
       </c>
       <c r="B28" t="s" s="2">
-        <v>297</v>
+        <v>293</v>
       </c>
       <c r="C28" s="2"/>
       <c r="D28" t="s" s="2">
@@ -5328,7 +5347,7 @@
         <v>81</v>
       </c>
       <c r="G28" t="s" s="2">
-        <v>93</v>
+        <v>82</v>
       </c>
       <c r="H28" t="s" s="2">
         <v>94</v>
@@ -5337,19 +5356,19 @@
         <v>80</v>
       </c>
       <c r="J28" t="s" s="2">
-        <v>80</v>
+        <v>94</v>
       </c>
       <c r="K28" t="s" s="2">
-        <v>287</v>
+        <v>294</v>
       </c>
       <c r="L28" t="s" s="2">
-        <v>298</v>
+        <v>295</v>
       </c>
       <c r="M28" t="s" s="2">
-        <v>299</v>
+        <v>296</v>
       </c>
       <c r="N28" t="s" s="2">
-        <v>300</v>
+        <v>297</v>
       </c>
       <c r="O28" s="2"/>
       <c r="P28" t="s" s="2">
@@ -5399,13 +5418,13 @@
         <v>80</v>
       </c>
       <c r="AF28" t="s" s="2">
-        <v>297</v>
+        <v>293</v>
       </c>
       <c r="AG28" t="s" s="2">
         <v>81</v>
       </c>
       <c r="AH28" t="s" s="2">
-        <v>93</v>
+        <v>82</v>
       </c>
       <c r="AI28" t="s" s="2">
         <v>80</v>
@@ -5414,33 +5433,33 @@
         <v>105</v>
       </c>
       <c r="AK28" t="s" s="2">
-        <v>291</v>
+        <v>298</v>
       </c>
       <c r="AL28" t="s" s="2">
+        <v>299</v>
+      </c>
+      <c r="AM28" t="s" s="2">
+        <v>300</v>
+      </c>
+      <c r="AN28" t="s" s="2">
         <v>301</v>
       </c>
-      <c r="AM28" t="s" s="2">
+      <c r="AO28" t="s" s="2">
+        <v>80</v>
+      </c>
+      <c r="AP28" t="s" s="2">
         <v>302</v>
       </c>
-      <c r="AN28" t="s" s="2">
+      <c r="AQ28" t="s" s="2">
         <v>303</v>
       </c>
-      <c r="AO28" t="s" s="2">
+    </row>
+    <row r="29">
+      <c r="A29" t="s" s="2">
         <v>304</v>
       </c>
-      <c r="AP28" t="s" s="2">
-        <v>305</v>
-      </c>
-      <c r="AQ28" t="s" s="2">
-        <v>306</v>
-      </c>
-    </row>
-    <row r="29" hidden="true">
-      <c r="A29" t="s" s="2">
-        <v>307</v>
-      </c>
       <c r="B29" t="s" s="2">
-        <v>307</v>
+        <v>304</v>
       </c>
       <c r="C29" s="2"/>
       <c r="D29" t="s" s="2">
@@ -5454,7 +5473,7 @@
         <v>93</v>
       </c>
       <c r="H29" t="s" s="2">
-        <v>80</v>
+        <v>94</v>
       </c>
       <c r="I29" t="s" s="2">
         <v>80</v>
@@ -5463,16 +5482,16 @@
         <v>80</v>
       </c>
       <c r="K29" t="s" s="2">
-        <v>308</v>
+        <v>294</v>
       </c>
       <c r="L29" t="s" s="2">
-        <v>309</v>
+        <v>305</v>
       </c>
       <c r="M29" t="s" s="2">
-        <v>310</v>
+        <v>306</v>
       </c>
       <c r="N29" t="s" s="2">
-        <v>311</v>
+        <v>307</v>
       </c>
       <c r="O29" s="2"/>
       <c r="P29" t="s" s="2">
@@ -5522,7 +5541,7 @@
         <v>80</v>
       </c>
       <c r="AF29" t="s" s="2">
-        <v>307</v>
+        <v>304</v>
       </c>
       <c r="AG29" t="s" s="2">
         <v>81</v>
@@ -5537,25 +5556,25 @@
         <v>105</v>
       </c>
       <c r="AK29" t="s" s="2">
-        <v>291</v>
+        <v>298</v>
       </c>
       <c r="AL29" t="s" s="2">
+        <v>308</v>
+      </c>
+      <c r="AM29" t="s" s="2">
+        <v>309</v>
+      </c>
+      <c r="AN29" t="s" s="2">
+        <v>310</v>
+      </c>
+      <c r="AO29" t="s" s="2">
+        <v>311</v>
+      </c>
+      <c r="AP29" t="s" s="2">
         <v>312</v>
       </c>
-      <c r="AM29" t="s" s="2">
+      <c r="AQ29" t="s" s="2">
         <v>313</v>
-      </c>
-      <c r="AN29" t="s" s="2">
-        <v>80</v>
-      </c>
-      <c r="AO29" t="s" s="2">
-        <v>80</v>
-      </c>
-      <c r="AP29" t="s" s="2">
-        <v>80</v>
-      </c>
-      <c r="AQ29" t="s" s="2">
-        <v>80</v>
       </c>
     </row>
     <row r="30" hidden="true">
@@ -5574,7 +5593,7 @@
         <v>81</v>
       </c>
       <c r="G30" t="s" s="2">
-        <v>82</v>
+        <v>93</v>
       </c>
       <c r="H30" t="s" s="2">
         <v>80</v>
@@ -5583,7 +5602,7 @@
         <v>80</v>
       </c>
       <c r="J30" t="s" s="2">
-        <v>94</v>
+        <v>80</v>
       </c>
       <c r="K30" t="s" s="2">
         <v>315</v>
@@ -5651,7 +5670,7 @@
         <v>81</v>
       </c>
       <c r="AH30" t="s" s="2">
-        <v>82</v>
+        <v>93</v>
       </c>
       <c r="AI30" t="s" s="2">
         <v>80</v>
@@ -5660,7 +5679,7 @@
         <v>105</v>
       </c>
       <c r="AK30" t="s" s="2">
-        <v>80</v>
+        <v>298</v>
       </c>
       <c r="AL30" t="s" s="2">
         <v>319</v>
@@ -5678,15 +5697,15 @@
         <v>80</v>
       </c>
       <c r="AQ30" t="s" s="2">
-        <v>321</v>
+        <v>80</v>
       </c>
     </row>
     <row r="31" hidden="true">
       <c r="A31" t="s" s="2">
-        <v>322</v>
+        <v>321</v>
       </c>
       <c r="B31" t="s" s="2">
-        <v>322</v>
+        <v>321</v>
       </c>
       <c r="C31" s="2"/>
       <c r="D31" t="s" s="2">
@@ -5697,7 +5716,7 @@
         <v>81</v>
       </c>
       <c r="G31" t="s" s="2">
-        <v>93</v>
+        <v>82</v>
       </c>
       <c r="H31" t="s" s="2">
         <v>80</v>
@@ -5706,18 +5725,20 @@
         <v>80</v>
       </c>
       <c r="J31" t="s" s="2">
-        <v>80</v>
+        <v>94</v>
       </c>
       <c r="K31" t="s" s="2">
-        <v>107</v>
+        <v>322</v>
       </c>
       <c r="L31" t="s" s="2">
-        <v>108</v>
+        <v>323</v>
       </c>
       <c r="M31" t="s" s="2">
-        <v>109</v>
-      </c>
-      <c r="N31" s="2"/>
+        <v>324</v>
+      </c>
+      <c r="N31" t="s" s="2">
+        <v>325</v>
+      </c>
       <c r="O31" s="2"/>
       <c r="P31" t="s" s="2">
         <v>80</v>
@@ -5766,28 +5787,28 @@
         <v>80</v>
       </c>
       <c r="AF31" t="s" s="2">
-        <v>110</v>
+        <v>321</v>
       </c>
       <c r="AG31" t="s" s="2">
         <v>81</v>
       </c>
       <c r="AH31" t="s" s="2">
-        <v>93</v>
+        <v>82</v>
       </c>
       <c r="AI31" t="s" s="2">
         <v>80</v>
       </c>
       <c r="AJ31" t="s" s="2">
-        <v>80</v>
+        <v>105</v>
       </c>
       <c r="AK31" t="s" s="2">
         <v>80</v>
       </c>
       <c r="AL31" t="s" s="2">
-        <v>80</v>
+        <v>326</v>
       </c>
       <c r="AM31" t="s" s="2">
-        <v>111</v>
+        <v>327</v>
       </c>
       <c r="AN31" t="s" s="2">
         <v>80</v>
@@ -5799,26 +5820,26 @@
         <v>80</v>
       </c>
       <c r="AQ31" t="s" s="2">
-        <v>80</v>
+        <v>328</v>
       </c>
     </row>
     <row r="32" hidden="true">
       <c r="A32" t="s" s="2">
-        <v>323</v>
+        <v>329</v>
       </c>
       <c r="B32" t="s" s="2">
-        <v>323</v>
+        <v>329</v>
       </c>
       <c r="C32" s="2"/>
       <c r="D32" t="s" s="2">
-        <v>113</v>
+        <v>80</v>
       </c>
       <c r="E32" s="2"/>
       <c r="F32" t="s" s="2">
         <v>81</v>
       </c>
       <c r="G32" t="s" s="2">
-        <v>82</v>
+        <v>93</v>
       </c>
       <c r="H32" t="s" s="2">
         <v>80</v>
@@ -5830,17 +5851,15 @@
         <v>80</v>
       </c>
       <c r="K32" t="s" s="2">
-        <v>114</v>
+        <v>107</v>
       </c>
       <c r="L32" t="s" s="2">
-        <v>115</v>
+        <v>108</v>
       </c>
       <c r="M32" t="s" s="2">
-        <v>116</v>
-      </c>
-      <c r="N32" t="s" s="2">
-        <v>117</v>
-      </c>
+        <v>109</v>
+      </c>
+      <c r="N32" s="2"/>
       <c r="O32" s="2"/>
       <c r="P32" t="s" s="2">
         <v>80</v>
@@ -5889,19 +5908,19 @@
         <v>80</v>
       </c>
       <c r="AF32" t="s" s="2">
-        <v>121</v>
+        <v>110</v>
       </c>
       <c r="AG32" t="s" s="2">
         <v>81</v>
       </c>
       <c r="AH32" t="s" s="2">
-        <v>82</v>
+        <v>93</v>
       </c>
       <c r="AI32" t="s" s="2">
         <v>80</v>
       </c>
       <c r="AJ32" t="s" s="2">
-        <v>122</v>
+        <v>80</v>
       </c>
       <c r="AK32" t="s" s="2">
         <v>80</v>
@@ -5927,14 +5946,14 @@
     </row>
     <row r="33" hidden="true">
       <c r="A33" t="s" s="2">
-        <v>324</v>
+        <v>330</v>
       </c>
       <c r="B33" t="s" s="2">
-        <v>324</v>
+        <v>330</v>
       </c>
       <c r="C33" s="2"/>
       <c r="D33" t="s" s="2">
-        <v>325</v>
+        <v>113</v>
       </c>
       <c r="E33" s="2"/>
       <c r="F33" t="s" s="2">
@@ -5947,26 +5966,24 @@
         <v>80</v>
       </c>
       <c r="I33" t="s" s="2">
-        <v>94</v>
+        <v>80</v>
       </c>
       <c r="J33" t="s" s="2">
-        <v>94</v>
+        <v>80</v>
       </c>
       <c r="K33" t="s" s="2">
         <v>114</v>
       </c>
       <c r="L33" t="s" s="2">
-        <v>326</v>
+        <v>115</v>
       </c>
       <c r="M33" t="s" s="2">
-        <v>327</v>
+        <v>116</v>
       </c>
       <c r="N33" t="s" s="2">
         <v>117</v>
       </c>
-      <c r="O33" t="s" s="2">
-        <v>199</v>
-      </c>
+      <c r="O33" s="2"/>
       <c r="P33" t="s" s="2">
         <v>80</v>
       </c>
@@ -6014,7 +6031,7 @@
         <v>80</v>
       </c>
       <c r="AF33" t="s" s="2">
-        <v>328</v>
+        <v>121</v>
       </c>
       <c r="AG33" t="s" s="2">
         <v>81</v>
@@ -6035,7 +6052,7 @@
         <v>80</v>
       </c>
       <c r="AM33" t="s" s="2">
-        <v>192</v>
+        <v>111</v>
       </c>
       <c r="AN33" t="s" s="2">
         <v>80</v>
@@ -6052,44 +6069,46 @@
     </row>
     <row r="34" hidden="true">
       <c r="A34" t="s" s="2">
-        <v>329</v>
+        <v>331</v>
       </c>
       <c r="B34" t="s" s="2">
-        <v>329</v>
+        <v>331</v>
       </c>
       <c r="C34" s="2"/>
       <c r="D34" t="s" s="2">
-        <v>80</v>
+        <v>332</v>
       </c>
       <c r="E34" s="2"/>
       <c r="F34" t="s" s="2">
-        <v>93</v>
+        <v>81</v>
       </c>
       <c r="G34" t="s" s="2">
-        <v>93</v>
+        <v>82</v>
       </c>
       <c r="H34" t="s" s="2">
         <v>80</v>
       </c>
       <c r="I34" t="s" s="2">
-        <v>80</v>
+        <v>94</v>
       </c>
       <c r="J34" t="s" s="2">
         <v>94</v>
       </c>
       <c r="K34" t="s" s="2">
-        <v>169</v>
+        <v>114</v>
       </c>
       <c r="L34" t="s" s="2">
-        <v>330</v>
+        <v>333</v>
       </c>
       <c r="M34" t="s" s="2">
-        <v>331</v>
+        <v>334</v>
       </c>
       <c r="N34" t="s" s="2">
-        <v>332</v>
-      </c>
-      <c r="O34" s="2"/>
+        <v>117</v>
+      </c>
+      <c r="O34" t="s" s="2">
+        <v>206</v>
+      </c>
       <c r="P34" t="s" s="2">
         <v>80</v>
       </c>
@@ -6113,13 +6132,13 @@
         <v>80</v>
       </c>
       <c r="X34" t="s" s="2">
-        <v>224</v>
+        <v>80</v>
       </c>
       <c r="Y34" t="s" s="2">
-        <v>333</v>
+        <v>80</v>
       </c>
       <c r="Z34" t="s" s="2">
-        <v>334</v>
+        <v>80</v>
       </c>
       <c r="AA34" t="s" s="2">
         <v>80</v>
@@ -6137,28 +6156,28 @@
         <v>80</v>
       </c>
       <c r="AF34" t="s" s="2">
-        <v>329</v>
+        <v>335</v>
       </c>
       <c r="AG34" t="s" s="2">
-        <v>93</v>
+        <v>81</v>
       </c>
       <c r="AH34" t="s" s="2">
-        <v>93</v>
+        <v>82</v>
       </c>
       <c r="AI34" t="s" s="2">
         <v>80</v>
       </c>
       <c r="AJ34" t="s" s="2">
-        <v>105</v>
+        <v>122</v>
       </c>
       <c r="AK34" t="s" s="2">
         <v>80</v>
       </c>
       <c r="AL34" t="s" s="2">
-        <v>335</v>
+        <v>80</v>
       </c>
       <c r="AM34" t="s" s="2">
-        <v>336</v>
+        <v>192</v>
       </c>
       <c r="AN34" t="s" s="2">
         <v>80</v>
@@ -6170,15 +6189,15 @@
         <v>80</v>
       </c>
       <c r="AQ34" t="s" s="2">
-        <v>337</v>
+        <v>80</v>
       </c>
     </row>
     <row r="35" hidden="true">
       <c r="A35" t="s" s="2">
-        <v>338</v>
+        <v>336</v>
       </c>
       <c r="B35" t="s" s="2">
-        <v>338</v>
+        <v>336</v>
       </c>
       <c r="C35" s="2"/>
       <c r="D35" t="s" s="2">
@@ -6201,15 +6220,17 @@
         <v>94</v>
       </c>
       <c r="K35" t="s" s="2">
+        <v>169</v>
+      </c>
+      <c r="L35" t="s" s="2">
+        <v>337</v>
+      </c>
+      <c r="M35" t="s" s="2">
+        <v>338</v>
+      </c>
+      <c r="N35" t="s" s="2">
         <v>339</v>
       </c>
-      <c r="L35" t="s" s="2">
-        <v>340</v>
-      </c>
-      <c r="M35" t="s" s="2">
-        <v>341</v>
-      </c>
-      <c r="N35" s="2"/>
       <c r="O35" s="2"/>
       <c r="P35" t="s" s="2">
         <v>80</v>
@@ -6234,13 +6255,13 @@
         <v>80</v>
       </c>
       <c r="X35" t="s" s="2">
-        <v>80</v>
+        <v>231</v>
       </c>
       <c r="Y35" t="s" s="2">
-        <v>80</v>
+        <v>340</v>
       </c>
       <c r="Z35" t="s" s="2">
-        <v>80</v>
+        <v>341</v>
       </c>
       <c r="AA35" t="s" s="2">
         <v>80</v>
@@ -6258,7 +6279,7 @@
         <v>80</v>
       </c>
       <c r="AF35" t="s" s="2">
-        <v>338</v>
+        <v>336</v>
       </c>
       <c r="AG35" t="s" s="2">
         <v>93</v>
@@ -6307,7 +6328,7 @@
       </c>
       <c r="E36" s="2"/>
       <c r="F36" t="s" s="2">
-        <v>81</v>
+        <v>93</v>
       </c>
       <c r="G36" t="s" s="2">
         <v>93</v>
@@ -6322,20 +6343,16 @@
         <v>94</v>
       </c>
       <c r="K36" t="s" s="2">
-        <v>107</v>
+        <v>346</v>
       </c>
       <c r="L36" t="s" s="2">
-        <v>346</v>
+        <v>347</v>
       </c>
       <c r="M36" t="s" s="2">
-        <v>347</v>
-      </c>
-      <c r="N36" t="s" s="2">
         <v>348</v>
       </c>
-      <c r="O36" t="s" s="2">
-        <v>349</v>
-      </c>
+      <c r="N36" s="2"/>
+      <c r="O36" s="2"/>
       <c r="P36" t="s" s="2">
         <v>80</v>
       </c>
@@ -6386,7 +6403,7 @@
         <v>345</v>
       </c>
       <c r="AG36" t="s" s="2">
-        <v>81</v>
+        <v>93</v>
       </c>
       <c r="AH36" t="s" s="2">
         <v>93</v>
@@ -6401,7 +6418,7 @@
         <v>80</v>
       </c>
       <c r="AL36" t="s" s="2">
-        <v>80</v>
+        <v>349</v>
       </c>
       <c r="AM36" t="s" s="2">
         <v>350</v>
@@ -6413,18 +6430,18 @@
         <v>80</v>
       </c>
       <c r="AP36" t="s" s="2">
+        <v>80</v>
+      </c>
+      <c r="AQ36" t="s" s="2">
         <v>351</v>
-      </c>
-      <c r="AQ36" t="s" s="2">
-        <v>352</v>
       </c>
     </row>
     <row r="37" hidden="true">
       <c r="A37" t="s" s="2">
-        <v>353</v>
+        <v>352</v>
       </c>
       <c r="B37" t="s" s="2">
-        <v>353</v>
+        <v>352</v>
       </c>
       <c r="C37" s="2"/>
       <c r="D37" t="s" s="2">
@@ -6435,7 +6452,7 @@
         <v>81</v>
       </c>
       <c r="G37" t="s" s="2">
-        <v>82</v>
+        <v>93</v>
       </c>
       <c r="H37" t="s" s="2">
         <v>80</v>
@@ -6447,19 +6464,19 @@
         <v>94</v>
       </c>
       <c r="K37" t="s" s="2">
-        <v>242</v>
+        <v>107</v>
       </c>
       <c r="L37" t="s" s="2">
+        <v>353</v>
+      </c>
+      <c r="M37" t="s" s="2">
         <v>354</v>
       </c>
-      <c r="M37" t="s" s="2">
+      <c r="N37" t="s" s="2">
         <v>355</v>
       </c>
-      <c r="N37" t="s" s="2">
+      <c r="O37" t="s" s="2">
         <v>356</v>
-      </c>
-      <c r="O37" t="s" s="2">
-        <v>357</v>
       </c>
       <c r="P37" t="s" s="2">
         <v>80</v>
@@ -6484,13 +6501,13 @@
         <v>80</v>
       </c>
       <c r="X37" t="s" s="2">
-        <v>151</v>
+        <v>80</v>
       </c>
       <c r="Y37" t="s" s="2">
-        <v>152</v>
+        <v>80</v>
       </c>
       <c r="Z37" t="s" s="2">
-        <v>153</v>
+        <v>80</v>
       </c>
       <c r="AA37" t="s" s="2">
         <v>80</v>
@@ -6508,13 +6525,13 @@
         <v>80</v>
       </c>
       <c r="AF37" t="s" s="2">
-        <v>353</v>
+        <v>352</v>
       </c>
       <c r="AG37" t="s" s="2">
         <v>81</v>
       </c>
       <c r="AH37" t="s" s="2">
-        <v>82</v>
+        <v>93</v>
       </c>
       <c r="AI37" t="s" s="2">
         <v>80</v>
@@ -6526,30 +6543,30 @@
         <v>80</v>
       </c>
       <c r="AL37" t="s" s="2">
+        <v>80</v>
+      </c>
+      <c r="AM37" t="s" s="2">
+        <v>357</v>
+      </c>
+      <c r="AN37" t="s" s="2">
+        <v>80</v>
+      </c>
+      <c r="AO37" t="s" s="2">
+        <v>80</v>
+      </c>
+      <c r="AP37" t="s" s="2">
         <v>358</v>
       </c>
-      <c r="AM37" t="s" s="2">
+      <c r="AQ37" t="s" s="2">
         <v>359</v>
       </c>
-      <c r="AN37" t="s" s="2">
+    </row>
+    <row r="38" hidden="true">
+      <c r="A38" t="s" s="2">
         <v>360</v>
       </c>
-      <c r="AO37" t="s" s="2">
-        <v>80</v>
-      </c>
-      <c r="AP37" t="s" s="2">
-        <v>361</v>
-      </c>
-      <c r="AQ37" t="s" s="2">
-        <v>362</v>
-      </c>
-    </row>
-    <row r="38">
-      <c r="A38" t="s" s="2">
-        <v>363</v>
-      </c>
       <c r="B38" t="s" s="2">
-        <v>363</v>
+        <v>360</v>
       </c>
       <c r="C38" s="2"/>
       <c r="D38" t="s" s="2">
@@ -6557,13 +6574,13 @@
       </c>
       <c r="E38" s="2"/>
       <c r="F38" t="s" s="2">
-        <v>93</v>
+        <v>81</v>
       </c>
       <c r="G38" t="s" s="2">
         <v>82</v>
       </c>
       <c r="H38" t="s" s="2">
-        <v>94</v>
+        <v>80</v>
       </c>
       <c r="I38" t="s" s="2">
         <v>80</v>
@@ -6572,16 +6589,20 @@
         <v>94</v>
       </c>
       <c r="K38" t="s" s="2">
-        <v>315</v>
+        <v>249</v>
       </c>
       <c r="L38" t="s" s="2">
+        <v>361</v>
+      </c>
+      <c r="M38" t="s" s="2">
+        <v>362</v>
+      </c>
+      <c r="N38" t="s" s="2">
+        <v>363</v>
+      </c>
+      <c r="O38" t="s" s="2">
         <v>364</v>
       </c>
-      <c r="M38" t="s" s="2">
-        <v>365</v>
-      </c>
-      <c r="N38" s="2"/>
-      <c r="O38" s="2"/>
       <c r="P38" t="s" s="2">
         <v>80</v>
       </c>
@@ -6605,13 +6626,13 @@
         <v>80</v>
       </c>
       <c r="X38" t="s" s="2">
-        <v>80</v>
+        <v>151</v>
       </c>
       <c r="Y38" t="s" s="2">
-        <v>80</v>
+        <v>152</v>
       </c>
       <c r="Z38" t="s" s="2">
-        <v>80</v>
+        <v>153</v>
       </c>
       <c r="AA38" t="s" s="2">
         <v>80</v>
@@ -6629,10 +6650,10 @@
         <v>80</v>
       </c>
       <c r="AF38" t="s" s="2">
-        <v>363</v>
+        <v>360</v>
       </c>
       <c r="AG38" t="s" s="2">
-        <v>93</v>
+        <v>81</v>
       </c>
       <c r="AH38" t="s" s="2">
         <v>82</v>
@@ -6647,30 +6668,30 @@
         <v>80</v>
       </c>
       <c r="AL38" t="s" s="2">
+        <v>365</v>
+      </c>
+      <c r="AM38" t="s" s="2">
         <v>366</v>
       </c>
-      <c r="AM38" t="s" s="2">
+      <c r="AN38" t="s" s="2">
         <v>367</v>
       </c>
-      <c r="AN38" t="s" s="2">
-        <v>80</v>
-      </c>
       <c r="AO38" t="s" s="2">
         <v>80</v>
       </c>
       <c r="AP38" t="s" s="2">
-        <v>80</v>
+        <v>368</v>
       </c>
       <c r="AQ38" t="s" s="2">
-        <v>80</v>
+        <v>369</v>
       </c>
     </row>
-    <row r="39" hidden="true">
+    <row r="39">
       <c r="A39" t="s" s="2">
-        <v>368</v>
+        <v>370</v>
       </c>
       <c r="B39" t="s" s="2">
-        <v>368</v>
+        <v>370</v>
       </c>
       <c r="C39" s="2"/>
       <c r="D39" t="s" s="2">
@@ -6678,28 +6699,28 @@
       </c>
       <c r="E39" s="2"/>
       <c r="F39" t="s" s="2">
-        <v>81</v>
+        <v>93</v>
       </c>
       <c r="G39" t="s" s="2">
-        <v>93</v>
+        <v>82</v>
       </c>
       <c r="H39" t="s" s="2">
-        <v>80</v>
+        <v>94</v>
       </c>
       <c r="I39" t="s" s="2">
         <v>80</v>
       </c>
       <c r="J39" t="s" s="2">
-        <v>80</v>
+        <v>94</v>
       </c>
       <c r="K39" t="s" s="2">
-        <v>107</v>
+        <v>322</v>
       </c>
       <c r="L39" t="s" s="2">
-        <v>108</v>
+        <v>371</v>
       </c>
       <c r="M39" t="s" s="2">
-        <v>109</v>
+        <v>372</v>
       </c>
       <c r="N39" s="2"/>
       <c r="O39" s="2"/>
@@ -6750,28 +6771,28 @@
         <v>80</v>
       </c>
       <c r="AF39" t="s" s="2">
-        <v>110</v>
+        <v>370</v>
       </c>
       <c r="AG39" t="s" s="2">
-        <v>81</v>
+        <v>93</v>
       </c>
       <c r="AH39" t="s" s="2">
-        <v>93</v>
+        <v>82</v>
       </c>
       <c r="AI39" t="s" s="2">
         <v>80</v>
       </c>
       <c r="AJ39" t="s" s="2">
-        <v>80</v>
+        <v>105</v>
       </c>
       <c r="AK39" t="s" s="2">
         <v>80</v>
       </c>
       <c r="AL39" t="s" s="2">
-        <v>80</v>
+        <v>373</v>
       </c>
       <c r="AM39" t="s" s="2">
-        <v>111</v>
+        <v>374</v>
       </c>
       <c r="AN39" t="s" s="2">
         <v>80</v>
@@ -6788,21 +6809,21 @@
     </row>
     <row r="40" hidden="true">
       <c r="A40" t="s" s="2">
-        <v>369</v>
+        <v>375</v>
       </c>
       <c r="B40" t="s" s="2">
-        <v>369</v>
+        <v>375</v>
       </c>
       <c r="C40" s="2"/>
       <c r="D40" t="s" s="2">
-        <v>113</v>
+        <v>80</v>
       </c>
       <c r="E40" s="2"/>
       <c r="F40" t="s" s="2">
         <v>81</v>
       </c>
       <c r="G40" t="s" s="2">
-        <v>82</v>
+        <v>93</v>
       </c>
       <c r="H40" t="s" s="2">
         <v>80</v>
@@ -6814,17 +6835,15 @@
         <v>80</v>
       </c>
       <c r="K40" t="s" s="2">
-        <v>114</v>
+        <v>107</v>
       </c>
       <c r="L40" t="s" s="2">
-        <v>115</v>
+        <v>108</v>
       </c>
       <c r="M40" t="s" s="2">
-        <v>116</v>
-      </c>
-      <c r="N40" t="s" s="2">
-        <v>117</v>
-      </c>
+        <v>109</v>
+      </c>
+      <c r="N40" s="2"/>
       <c r="O40" s="2"/>
       <c r="P40" t="s" s="2">
         <v>80</v>
@@ -6873,19 +6892,19 @@
         <v>80</v>
       </c>
       <c r="AF40" t="s" s="2">
-        <v>121</v>
+        <v>110</v>
       </c>
       <c r="AG40" t="s" s="2">
         <v>81</v>
       </c>
       <c r="AH40" t="s" s="2">
-        <v>82</v>
+        <v>93</v>
       </c>
       <c r="AI40" t="s" s="2">
         <v>80</v>
       </c>
       <c r="AJ40" t="s" s="2">
-        <v>122</v>
+        <v>80</v>
       </c>
       <c r="AK40" t="s" s="2">
         <v>80</v>
@@ -6911,14 +6930,14 @@
     </row>
     <row r="41" hidden="true">
       <c r="A41" t="s" s="2">
-        <v>370</v>
+        <v>376</v>
       </c>
       <c r="B41" t="s" s="2">
-        <v>370</v>
+        <v>376</v>
       </c>
       <c r="C41" s="2"/>
       <c r="D41" t="s" s="2">
-        <v>325</v>
+        <v>113</v>
       </c>
       <c r="E41" s="2"/>
       <c r="F41" t="s" s="2">
@@ -6931,26 +6950,24 @@
         <v>80</v>
       </c>
       <c r="I41" t="s" s="2">
-        <v>94</v>
+        <v>80</v>
       </c>
       <c r="J41" t="s" s="2">
-        <v>94</v>
+        <v>80</v>
       </c>
       <c r="K41" t="s" s="2">
         <v>114</v>
       </c>
       <c r="L41" t="s" s="2">
-        <v>326</v>
+        <v>115</v>
       </c>
       <c r="M41" t="s" s="2">
-        <v>327</v>
+        <v>116</v>
       </c>
       <c r="N41" t="s" s="2">
         <v>117</v>
       </c>
-      <c r="O41" t="s" s="2">
-        <v>199</v>
-      </c>
+      <c r="O41" s="2"/>
       <c r="P41" t="s" s="2">
         <v>80</v>
       </c>
@@ -6998,7 +7015,7 @@
         <v>80</v>
       </c>
       <c r="AF41" t="s" s="2">
-        <v>328</v>
+        <v>121</v>
       </c>
       <c r="AG41" t="s" s="2">
         <v>81</v>
@@ -7019,7 +7036,7 @@
         <v>80</v>
       </c>
       <c r="AM41" t="s" s="2">
-        <v>192</v>
+        <v>111</v>
       </c>
       <c r="AN41" t="s" s="2">
         <v>80</v>
@@ -7034,44 +7051,48 @@
         <v>80</v>
       </c>
     </row>
-    <row r="42">
+    <row r="42" hidden="true">
       <c r="A42" t="s" s="2">
-        <v>371</v>
+        <v>377</v>
       </c>
       <c r="B42" t="s" s="2">
-        <v>371</v>
+        <v>377</v>
       </c>
       <c r="C42" s="2"/>
       <c r="D42" t="s" s="2">
-        <v>80</v>
+        <v>332</v>
       </c>
       <c r="E42" s="2"/>
       <c r="F42" t="s" s="2">
-        <v>93</v>
+        <v>81</v>
       </c>
       <c r="G42" t="s" s="2">
-        <v>93</v>
+        <v>82</v>
       </c>
       <c r="H42" t="s" s="2">
+        <v>80</v>
+      </c>
+      <c r="I42" t="s" s="2">
         <v>94</v>
-      </c>
-      <c r="I42" t="s" s="2">
-        <v>80</v>
       </c>
       <c r="J42" t="s" s="2">
         <v>94</v>
       </c>
       <c r="K42" t="s" s="2">
-        <v>372</v>
+        <v>114</v>
       </c>
       <c r="L42" t="s" s="2">
-        <v>373</v>
+        <v>333</v>
       </c>
       <c r="M42" t="s" s="2">
-        <v>374</v>
-      </c>
-      <c r="N42" s="2"/>
-      <c r="O42" s="2"/>
+        <v>334</v>
+      </c>
+      <c r="N42" t="s" s="2">
+        <v>117</v>
+      </c>
+      <c r="O42" t="s" s="2">
+        <v>206</v>
+      </c>
       <c r="P42" t="s" s="2">
         <v>80</v>
       </c>
@@ -7119,48 +7140,48 @@
         <v>80</v>
       </c>
       <c r="AF42" t="s" s="2">
-        <v>371</v>
+        <v>335</v>
       </c>
       <c r="AG42" t="s" s="2">
-        <v>93</v>
+        <v>81</v>
       </c>
       <c r="AH42" t="s" s="2">
-        <v>93</v>
+        <v>82</v>
       </c>
       <c r="AI42" t="s" s="2">
         <v>80</v>
       </c>
       <c r="AJ42" t="s" s="2">
-        <v>105</v>
+        <v>122</v>
       </c>
       <c r="AK42" t="s" s="2">
         <v>80</v>
       </c>
       <c r="AL42" t="s" s="2">
-        <v>375</v>
+        <v>80</v>
       </c>
       <c r="AM42" t="s" s="2">
-        <v>367</v>
+        <v>192</v>
       </c>
       <c r="AN42" t="s" s="2">
-        <v>376</v>
+        <v>80</v>
       </c>
       <c r="AO42" t="s" s="2">
         <v>80</v>
       </c>
       <c r="AP42" t="s" s="2">
-        <v>377</v>
+        <v>80</v>
       </c>
       <c r="AQ42" t="s" s="2">
+        <v>80</v>
+      </c>
+    </row>
+    <row r="43">
+      <c r="A43" t="s" s="2">
         <v>378</v>
       </c>
-    </row>
-    <row r="43" hidden="true">
-      <c r="A43" t="s" s="2">
-        <v>379</v>
-      </c>
       <c r="B43" t="s" s="2">
-        <v>379</v>
+        <v>378</v>
       </c>
       <c r="C43" s="2"/>
       <c r="D43" t="s" s="2">
@@ -7168,28 +7189,28 @@
       </c>
       <c r="E43" s="2"/>
       <c r="F43" t="s" s="2">
-        <v>81</v>
+        <v>93</v>
       </c>
       <c r="G43" t="s" s="2">
         <v>93</v>
       </c>
       <c r="H43" t="s" s="2">
-        <v>80</v>
+        <v>94</v>
       </c>
       <c r="I43" t="s" s="2">
         <v>80</v>
       </c>
       <c r="J43" t="s" s="2">
-        <v>80</v>
+        <v>94</v>
       </c>
       <c r="K43" t="s" s="2">
-        <v>107</v>
+        <v>379</v>
       </c>
       <c r="L43" t="s" s="2">
-        <v>108</v>
+        <v>380</v>
       </c>
       <c r="M43" t="s" s="2">
-        <v>109</v>
+        <v>381</v>
       </c>
       <c r="N43" s="2"/>
       <c r="O43" s="2"/>
@@ -7240,10 +7261,10 @@
         <v>80</v>
       </c>
       <c r="AF43" t="s" s="2">
-        <v>110</v>
+        <v>378</v>
       </c>
       <c r="AG43" t="s" s="2">
-        <v>81</v>
+        <v>93</v>
       </c>
       <c r="AH43" t="s" s="2">
         <v>93</v>
@@ -7252,47 +7273,47 @@
         <v>80</v>
       </c>
       <c r="AJ43" t="s" s="2">
-        <v>80</v>
+        <v>105</v>
       </c>
       <c r="AK43" t="s" s="2">
         <v>80</v>
       </c>
       <c r="AL43" t="s" s="2">
-        <v>80</v>
+        <v>382</v>
       </c>
       <c r="AM43" t="s" s="2">
-        <v>111</v>
+        <v>374</v>
       </c>
       <c r="AN43" t="s" s="2">
-        <v>80</v>
+        <v>383</v>
       </c>
       <c r="AO43" t="s" s="2">
         <v>80</v>
       </c>
       <c r="AP43" t="s" s="2">
-        <v>80</v>
+        <v>384</v>
       </c>
       <c r="AQ43" t="s" s="2">
-        <v>80</v>
+        <v>385</v>
       </c>
     </row>
     <row r="44" hidden="true">
       <c r="A44" t="s" s="2">
-        <v>380</v>
+        <v>386</v>
       </c>
       <c r="B44" t="s" s="2">
-        <v>380</v>
+        <v>386</v>
       </c>
       <c r="C44" s="2"/>
       <c r="D44" t="s" s="2">
-        <v>113</v>
+        <v>80</v>
       </c>
       <c r="E44" s="2"/>
       <c r="F44" t="s" s="2">
         <v>81</v>
       </c>
       <c r="G44" t="s" s="2">
-        <v>82</v>
+        <v>93</v>
       </c>
       <c r="H44" t="s" s="2">
         <v>80</v>
@@ -7304,17 +7325,15 @@
         <v>80</v>
       </c>
       <c r="K44" t="s" s="2">
-        <v>114</v>
+        <v>107</v>
       </c>
       <c r="L44" t="s" s="2">
-        <v>115</v>
+        <v>108</v>
       </c>
       <c r="M44" t="s" s="2">
-        <v>116</v>
-      </c>
-      <c r="N44" t="s" s="2">
-        <v>117</v>
-      </c>
+        <v>109</v>
+      </c>
+      <c r="N44" s="2"/>
       <c r="O44" s="2"/>
       <c r="P44" t="s" s="2">
         <v>80</v>
@@ -7351,31 +7370,31 @@
         <v>80</v>
       </c>
       <c r="AB44" t="s" s="2">
-        <v>118</v>
+        <v>80</v>
       </c>
       <c r="AC44" t="s" s="2">
-        <v>119</v>
+        <v>80</v>
       </c>
       <c r="AD44" t="s" s="2">
         <v>80</v>
       </c>
       <c r="AE44" t="s" s="2">
-        <v>120</v>
+        <v>80</v>
       </c>
       <c r="AF44" t="s" s="2">
-        <v>121</v>
+        <v>110</v>
       </c>
       <c r="AG44" t="s" s="2">
         <v>81</v>
       </c>
       <c r="AH44" t="s" s="2">
-        <v>82</v>
+        <v>93</v>
       </c>
       <c r="AI44" t="s" s="2">
         <v>80</v>
       </c>
       <c r="AJ44" t="s" s="2">
-        <v>122</v>
+        <v>80</v>
       </c>
       <c r="AK44" t="s" s="2">
         <v>80</v>
@@ -7399,46 +7418,46 @@
         <v>80</v>
       </c>
     </row>
-    <row r="45">
+    <row r="45" hidden="true">
       <c r="A45" t="s" s="2">
-        <v>381</v>
+        <v>387</v>
       </c>
       <c r="B45" t="s" s="2">
-        <v>381</v>
+        <v>387</v>
       </c>
       <c r="C45" s="2"/>
       <c r="D45" t="s" s="2">
-        <v>80</v>
+        <v>113</v>
       </c>
       <c r="E45" s="2"/>
       <c r="F45" t="s" s="2">
         <v>81</v>
       </c>
       <c r="G45" t="s" s="2">
-        <v>93</v>
+        <v>82</v>
       </c>
       <c r="H45" t="s" s="2">
-        <v>94</v>
+        <v>80</v>
       </c>
       <c r="I45" t="s" s="2">
         <v>80</v>
       </c>
       <c r="J45" t="s" s="2">
-        <v>94</v>
+        <v>80</v>
       </c>
       <c r="K45" t="s" s="2">
-        <v>169</v>
+        <v>114</v>
       </c>
       <c r="L45" t="s" s="2">
-        <v>382</v>
+        <v>115</v>
       </c>
       <c r="M45" t="s" s="2">
-        <v>383</v>
-      </c>
-      <c r="N45" s="2"/>
-      <c r="O45" t="s" s="2">
-        <v>384</v>
-      </c>
+        <v>116</v>
+      </c>
+      <c r="N45" t="s" s="2">
+        <v>117</v>
+      </c>
+      <c r="O45" s="2"/>
       <c r="P45" t="s" s="2">
         <v>80</v>
       </c>
@@ -7450,7 +7469,7 @@
         <v>80</v>
       </c>
       <c r="T45" t="s" s="2">
-        <v>385</v>
+        <v>80</v>
       </c>
       <c r="U45" t="s" s="2">
         <v>80</v>
@@ -7462,72 +7481,72 @@
         <v>80</v>
       </c>
       <c r="X45" t="s" s="2">
-        <v>224</v>
+        <v>80</v>
       </c>
       <c r="Y45" t="s" s="2">
-        <v>386</v>
+        <v>80</v>
       </c>
       <c r="Z45" t="s" s="2">
-        <v>387</v>
+        <v>80</v>
       </c>
       <c r="AA45" t="s" s="2">
         <v>80</v>
       </c>
       <c r="AB45" t="s" s="2">
-        <v>80</v>
+        <v>118</v>
       </c>
       <c r="AC45" t="s" s="2">
-        <v>80</v>
+        <v>119</v>
       </c>
       <c r="AD45" t="s" s="2">
         <v>80</v>
       </c>
       <c r="AE45" t="s" s="2">
-        <v>80</v>
+        <v>120</v>
       </c>
       <c r="AF45" t="s" s="2">
+        <v>121</v>
+      </c>
+      <c r="AG45" t="s" s="2">
+        <v>81</v>
+      </c>
+      <c r="AH45" t="s" s="2">
+        <v>82</v>
+      </c>
+      <c r="AI45" t="s" s="2">
+        <v>80</v>
+      </c>
+      <c r="AJ45" t="s" s="2">
+        <v>122</v>
+      </c>
+      <c r="AK45" t="s" s="2">
+        <v>80</v>
+      </c>
+      <c r="AL45" t="s" s="2">
+        <v>80</v>
+      </c>
+      <c r="AM45" t="s" s="2">
+        <v>111</v>
+      </c>
+      <c r="AN45" t="s" s="2">
+        <v>80</v>
+      </c>
+      <c r="AO45" t="s" s="2">
+        <v>80</v>
+      </c>
+      <c r="AP45" t="s" s="2">
+        <v>80</v>
+      </c>
+      <c r="AQ45" t="s" s="2">
+        <v>80</v>
+      </c>
+    </row>
+    <row r="46">
+      <c r="A46" t="s" s="2">
         <v>388</v>
       </c>
-      <c r="AG45" t="s" s="2">
-        <v>81</v>
-      </c>
-      <c r="AH45" t="s" s="2">
-        <v>93</v>
-      </c>
-      <c r="AI45" t="s" s="2">
-        <v>80</v>
-      </c>
-      <c r="AJ45" t="s" s="2">
-        <v>105</v>
-      </c>
-      <c r="AK45" t="s" s="2">
-        <v>80</v>
-      </c>
-      <c r="AL45" t="s" s="2">
-        <v>80</v>
-      </c>
-      <c r="AM45" t="s" s="2">
-        <v>389</v>
-      </c>
-      <c r="AN45" t="s" s="2">
-        <v>80</v>
-      </c>
-      <c r="AO45" t="s" s="2">
-        <v>80</v>
-      </c>
-      <c r="AP45" t="s" s="2">
-        <v>390</v>
-      </c>
-      <c r="AQ45" t="s" s="2">
-        <v>80</v>
-      </c>
-    </row>
-    <row r="46" hidden="true">
-      <c r="A46" t="s" s="2">
-        <v>391</v>
-      </c>
       <c r="B46" t="s" s="2">
-        <v>391</v>
+        <v>388</v>
       </c>
       <c r="C46" s="2"/>
       <c r="D46" t="s" s="2">
@@ -7541,7 +7560,7 @@
         <v>93</v>
       </c>
       <c r="H46" t="s" s="2">
-        <v>80</v>
+        <v>94</v>
       </c>
       <c r="I46" t="s" s="2">
         <v>80</v>
@@ -7553,14 +7572,14 @@
         <v>169</v>
       </c>
       <c r="L46" t="s" s="2">
-        <v>392</v>
+        <v>389</v>
       </c>
       <c r="M46" t="s" s="2">
-        <v>393</v>
+        <v>390</v>
       </c>
       <c r="N46" s="2"/>
       <c r="O46" t="s" s="2">
-        <v>394</v>
+        <v>391</v>
       </c>
       <c r="P46" t="s" s="2">
         <v>80</v>
@@ -7573,43 +7592,43 @@
         <v>80</v>
       </c>
       <c r="T46" t="s" s="2">
+        <v>392</v>
+      </c>
+      <c r="U46" t="s" s="2">
+        <v>80</v>
+      </c>
+      <c r="V46" t="s" s="2">
+        <v>80</v>
+      </c>
+      <c r="W46" t="s" s="2">
+        <v>80</v>
+      </c>
+      <c r="X46" t="s" s="2">
+        <v>231</v>
+      </c>
+      <c r="Y46" t="s" s="2">
+        <v>393</v>
+      </c>
+      <c r="Z46" t="s" s="2">
+        <v>394</v>
+      </c>
+      <c r="AA46" t="s" s="2">
+        <v>80</v>
+      </c>
+      <c r="AB46" t="s" s="2">
+        <v>80</v>
+      </c>
+      <c r="AC46" t="s" s="2">
+        <v>80</v>
+      </c>
+      <c r="AD46" t="s" s="2">
+        <v>80</v>
+      </c>
+      <c r="AE46" t="s" s="2">
+        <v>80</v>
+      </c>
+      <c r="AF46" t="s" s="2">
         <v>395</v>
-      </c>
-      <c r="U46" t="s" s="2">
-        <v>80</v>
-      </c>
-      <c r="V46" t="s" s="2">
-        <v>80</v>
-      </c>
-      <c r="W46" t="s" s="2">
-        <v>80</v>
-      </c>
-      <c r="X46" t="s" s="2">
-        <v>173</v>
-      </c>
-      <c r="Y46" t="s" s="2">
-        <v>174</v>
-      </c>
-      <c r="Z46" t="s" s="2">
-        <v>175</v>
-      </c>
-      <c r="AA46" t="s" s="2">
-        <v>80</v>
-      </c>
-      <c r="AB46" t="s" s="2">
-        <v>80</v>
-      </c>
-      <c r="AC46" t="s" s="2">
-        <v>80</v>
-      </c>
-      <c r="AD46" t="s" s="2">
-        <v>80</v>
-      </c>
-      <c r="AE46" t="s" s="2">
-        <v>80</v>
-      </c>
-      <c r="AF46" t="s" s="2">
-        <v>396</v>
       </c>
       <c r="AG46" t="s" s="2">
         <v>81</v>
@@ -7630,22 +7649,22 @@
         <v>80</v>
       </c>
       <c r="AM46" t="s" s="2">
+        <v>396</v>
+      </c>
+      <c r="AN46" t="s" s="2">
+        <v>80</v>
+      </c>
+      <c r="AO46" t="s" s="2">
+        <v>80</v>
+      </c>
+      <c r="AP46" t="s" s="2">
         <v>397</v>
       </c>
-      <c r="AN46" t="s" s="2">
-        <v>80</v>
-      </c>
-      <c r="AO46" t="s" s="2">
-        <v>80</v>
-      </c>
-      <c r="AP46" t="s" s="2">
-        <v>80</v>
-      </c>
       <c r="AQ46" t="s" s="2">
         <v>80</v>
       </c>
     </row>
-    <row r="47">
+    <row r="47" hidden="true">
       <c r="A47" t="s" s="2">
         <v>398</v>
       </c>
@@ -7664,28 +7683,26 @@
         <v>93</v>
       </c>
       <c r="H47" t="s" s="2">
+        <v>80</v>
+      </c>
+      <c r="I47" t="s" s="2">
+        <v>80</v>
+      </c>
+      <c r="J47" t="s" s="2">
         <v>94</v>
       </c>
-      <c r="I47" t="s" s="2">
-        <v>80</v>
-      </c>
-      <c r="J47" t="s" s="2">
-        <v>80</v>
-      </c>
       <c r="K47" t="s" s="2">
+        <v>169</v>
+      </c>
+      <c r="L47" t="s" s="2">
         <v>399</v>
       </c>
-      <c r="L47" t="s" s="2">
+      <c r="M47" t="s" s="2">
         <v>400</v>
       </c>
-      <c r="M47" t="s" s="2">
+      <c r="N47" s="2"/>
+      <c r="O47" t="s" s="2">
         <v>401</v>
-      </c>
-      <c r="N47" t="s" s="2">
-        <v>402</v>
-      </c>
-      <c r="O47" t="s" s="2">
-        <v>403</v>
       </c>
       <c r="P47" t="s" s="2">
         <v>80</v>
@@ -7698,7 +7715,7 @@
         <v>80</v>
       </c>
       <c r="T47" t="s" s="2">
-        <v>80</v>
+        <v>402</v>
       </c>
       <c r="U47" t="s" s="2">
         <v>80</v>
@@ -7710,13 +7727,13 @@
         <v>80</v>
       </c>
       <c r="X47" t="s" s="2">
-        <v>80</v>
+        <v>173</v>
       </c>
       <c r="Y47" t="s" s="2">
-        <v>80</v>
+        <v>174</v>
       </c>
       <c r="Z47" t="s" s="2">
-        <v>80</v>
+        <v>175</v>
       </c>
       <c r="AA47" t="s" s="2">
         <v>80</v>
@@ -7734,7 +7751,7 @@
         <v>80</v>
       </c>
       <c r="AF47" t="s" s="2">
-        <v>404</v>
+        <v>403</v>
       </c>
       <c r="AG47" t="s" s="2">
         <v>81</v>
@@ -7755,7 +7772,7 @@
         <v>80</v>
       </c>
       <c r="AM47" t="s" s="2">
-        <v>405</v>
+        <v>404</v>
       </c>
       <c r="AN47" t="s" s="2">
         <v>80</v>
@@ -7764,7 +7781,7 @@
         <v>80</v>
       </c>
       <c r="AP47" t="s" s="2">
-        <v>406</v>
+        <v>80</v>
       </c>
       <c r="AQ47" t="s" s="2">
         <v>80</v>
@@ -7772,10 +7789,10 @@
     </row>
     <row r="48">
       <c r="A48" t="s" s="2">
-        <v>407</v>
+        <v>405</v>
       </c>
       <c r="B48" t="s" s="2">
-        <v>407</v>
+        <v>405</v>
       </c>
       <c r="C48" s="2"/>
       <c r="D48" t="s" s="2">
@@ -7795,22 +7812,22 @@
         <v>80</v>
       </c>
       <c r="J48" t="s" s="2">
-        <v>94</v>
+        <v>80</v>
       </c>
       <c r="K48" t="s" s="2">
+        <v>406</v>
+      </c>
+      <c r="L48" t="s" s="2">
+        <v>407</v>
+      </c>
+      <c r="M48" t="s" s="2">
         <v>408</v>
       </c>
-      <c r="L48" t="s" s="2">
+      <c r="N48" t="s" s="2">
         <v>409</v>
       </c>
-      <c r="M48" t="s" s="2">
+      <c r="O48" t="s" s="2">
         <v>410</v>
-      </c>
-      <c r="N48" t="s" s="2">
-        <v>411</v>
-      </c>
-      <c r="O48" t="s" s="2">
-        <v>412</v>
       </c>
       <c r="P48" t="s" s="2">
         <v>80</v>
@@ -7823,7 +7840,7 @@
         <v>80</v>
       </c>
       <c r="T48" t="s" s="2">
-        <v>413</v>
+        <v>80</v>
       </c>
       <c r="U48" t="s" s="2">
         <v>80</v>
@@ -7859,7 +7876,7 @@
         <v>80</v>
       </c>
       <c r="AF48" t="s" s="2">
-        <v>414</v>
+        <v>411</v>
       </c>
       <c r="AG48" t="s" s="2">
         <v>81</v>
@@ -7880,7 +7897,7 @@
         <v>80</v>
       </c>
       <c r="AM48" t="s" s="2">
-        <v>415</v>
+        <v>412</v>
       </c>
       <c r="AN48" t="s" s="2">
         <v>80</v>
@@ -7889,18 +7906,18 @@
         <v>80</v>
       </c>
       <c r="AP48" t="s" s="2">
-        <v>416</v>
+        <v>413</v>
       </c>
       <c r="AQ48" t="s" s="2">
         <v>80</v>
       </c>
     </row>
-    <row r="49" hidden="true">
+    <row r="49">
       <c r="A49" t="s" s="2">
-        <v>417</v>
+        <v>414</v>
       </c>
       <c r="B49" t="s" s="2">
-        <v>417</v>
+        <v>414</v>
       </c>
       <c r="C49" s="2"/>
       <c r="D49" t="s" s="2">
@@ -7914,7 +7931,7 @@
         <v>93</v>
       </c>
       <c r="H49" t="s" s="2">
-        <v>80</v>
+        <v>94</v>
       </c>
       <c r="I49" t="s" s="2">
         <v>80</v>
@@ -7923,19 +7940,19 @@
         <v>94</v>
       </c>
       <c r="K49" t="s" s="2">
+        <v>415</v>
+      </c>
+      <c r="L49" t="s" s="2">
+        <v>416</v>
+      </c>
+      <c r="M49" t="s" s="2">
+        <v>417</v>
+      </c>
+      <c r="N49" t="s" s="2">
         <v>418</v>
       </c>
-      <c r="L49" t="s" s="2">
+      <c r="O49" t="s" s="2">
         <v>419</v>
-      </c>
-      <c r="M49" t="s" s="2">
-        <v>420</v>
-      </c>
-      <c r="N49" t="s" s="2">
-        <v>421</v>
-      </c>
-      <c r="O49" t="s" s="2">
-        <v>422</v>
       </c>
       <c r="P49" t="s" s="2">
         <v>80</v>
@@ -7948,7 +7965,7 @@
         <v>80</v>
       </c>
       <c r="T49" t="s" s="2">
-        <v>80</v>
+        <v>420</v>
       </c>
       <c r="U49" t="s" s="2">
         <v>80</v>
@@ -7984,7 +8001,7 @@
         <v>80</v>
       </c>
       <c r="AF49" t="s" s="2">
-        <v>423</v>
+        <v>421</v>
       </c>
       <c r="AG49" t="s" s="2">
         <v>81</v>
@@ -8005,7 +8022,7 @@
         <v>80</v>
       </c>
       <c r="AM49" t="s" s="2">
-        <v>424</v>
+        <v>422</v>
       </c>
       <c r="AN49" t="s" s="2">
         <v>80</v>
@@ -8014,7 +8031,7 @@
         <v>80</v>
       </c>
       <c r="AP49" t="s" s="2">
-        <v>80</v>
+        <v>423</v>
       </c>
       <c r="AQ49" t="s" s="2">
         <v>80</v>
@@ -8022,10 +8039,10 @@
     </row>
     <row r="50" hidden="true">
       <c r="A50" t="s" s="2">
-        <v>425</v>
+        <v>424</v>
       </c>
       <c r="B50" t="s" s="2">
-        <v>425</v>
+        <v>424</v>
       </c>
       <c r="C50" s="2"/>
       <c r="D50" t="s" s="2">
@@ -8048,7 +8065,7 @@
         <v>94</v>
       </c>
       <c r="K50" t="s" s="2">
-        <v>399</v>
+        <v>425</v>
       </c>
       <c r="L50" t="s" s="2">
         <v>426</v>
@@ -8145,7 +8162,7 @@
         <v>80</v>
       </c>
     </row>
-    <row r="51">
+    <row r="51" hidden="true">
       <c r="A51" t="s" s="2">
         <v>432</v>
       </c>
@@ -8164,7 +8181,7 @@
         <v>93</v>
       </c>
       <c r="H51" t="s" s="2">
-        <v>94</v>
+        <v>80</v>
       </c>
       <c r="I51" t="s" s="2">
         <v>80</v>
@@ -8173,7 +8190,7 @@
         <v>94</v>
       </c>
       <c r="K51" t="s" s="2">
-        <v>107</v>
+        <v>406</v>
       </c>
       <c r="L51" t="s" s="2">
         <v>433</v>
@@ -8181,9 +8198,11 @@
       <c r="M51" t="s" s="2">
         <v>434</v>
       </c>
-      <c r="N51" s="2"/>
+      <c r="N51" t="s" s="2">
+        <v>435</v>
+      </c>
       <c r="O51" t="s" s="2">
-        <v>435</v>
+        <v>436</v>
       </c>
       <c r="P51" t="s" s="2">
         <v>80</v>
@@ -8196,7 +8215,7 @@
         <v>80</v>
       </c>
       <c r="T51" t="s" s="2">
-        <v>436</v>
+        <v>80</v>
       </c>
       <c r="U51" t="s" s="2">
         <v>80</v>
@@ -8268,7 +8287,7 @@
         <v>80</v>
       </c>
     </row>
-    <row r="52" hidden="true">
+    <row r="52">
       <c r="A52" t="s" s="2">
         <v>439</v>
       </c>
@@ -8287,7 +8306,7 @@
         <v>93</v>
       </c>
       <c r="H52" t="s" s="2">
-        <v>80</v>
+        <v>94</v>
       </c>
       <c r="I52" t="s" s="2">
         <v>80</v>
@@ -8296,17 +8315,17 @@
         <v>94</v>
       </c>
       <c r="K52" t="s" s="2">
+        <v>107</v>
+      </c>
+      <c r="L52" t="s" s="2">
         <v>440</v>
       </c>
-      <c r="L52" t="s" s="2">
+      <c r="M52" t="s" s="2">
         <v>441</v>
-      </c>
-      <c r="M52" t="s" s="2">
-        <v>442</v>
       </c>
       <c r="N52" s="2"/>
       <c r="O52" t="s" s="2">
-        <v>443</v>
+        <v>442</v>
       </c>
       <c r="P52" t="s" s="2">
         <v>80</v>
@@ -8319,7 +8338,7 @@
         <v>80</v>
       </c>
       <c r="T52" t="s" s="2">
-        <v>80</v>
+        <v>443</v>
       </c>
       <c r="U52" t="s" s="2">
         <v>80</v>
@@ -8376,7 +8395,7 @@
         <v>80</v>
       </c>
       <c r="AM52" t="s" s="2">
-        <v>424</v>
+        <v>445</v>
       </c>
       <c r="AN52" t="s" s="2">
         <v>80</v>
@@ -8393,10 +8412,10 @@
     </row>
     <row r="53" hidden="true">
       <c r="A53" t="s" s="2">
-        <v>445</v>
+        <v>446</v>
       </c>
       <c r="B53" t="s" s="2">
-        <v>445</v>
+        <v>446</v>
       </c>
       <c r="C53" s="2"/>
       <c r="D53" t="s" s="2">
@@ -8419,18 +8438,18 @@
         <v>94</v>
       </c>
       <c r="K53" t="s" s="2">
-        <v>147</v>
+        <v>447</v>
       </c>
       <c r="L53" t="s" s="2">
-        <v>446</v>
+        <v>448</v>
       </c>
       <c r="M53" t="s" s="2">
-        <v>447</v>
-      </c>
-      <c r="N53" t="s" s="2">
-        <v>448</v>
-      </c>
-      <c r="O53" s="2"/>
+        <v>449</v>
+      </c>
+      <c r="N53" s="2"/>
+      <c r="O53" t="s" s="2">
+        <v>450</v>
+      </c>
       <c r="P53" t="s" s="2">
         <v>80</v>
       </c>
@@ -8454,13 +8473,13 @@
         <v>80</v>
       </c>
       <c r="X53" t="s" s="2">
-        <v>173</v>
+        <v>80</v>
       </c>
       <c r="Y53" t="s" s="2">
-        <v>449</v>
+        <v>80</v>
       </c>
       <c r="Z53" t="s" s="2">
-        <v>450</v>
+        <v>80</v>
       </c>
       <c r="AA53" t="s" s="2">
         <v>80</v>
@@ -8478,7 +8497,7 @@
         <v>80</v>
       </c>
       <c r="AF53" t="s" s="2">
-        <v>445</v>
+        <v>451</v>
       </c>
       <c r="AG53" t="s" s="2">
         <v>81</v>
@@ -8496,30 +8515,30 @@
         <v>80</v>
       </c>
       <c r="AL53" t="s" s="2">
-        <v>451</v>
+        <v>80</v>
       </c>
       <c r="AM53" t="s" s="2">
-        <v>367</v>
+        <v>431</v>
       </c>
       <c r="AN53" t="s" s="2">
+        <v>80</v>
+      </c>
+      <c r="AO53" t="s" s="2">
+        <v>80</v>
+      </c>
+      <c r="AP53" t="s" s="2">
+        <v>80</v>
+      </c>
+      <c r="AQ53" t="s" s="2">
+        <v>80</v>
+      </c>
+    </row>
+    <row r="54" hidden="true">
+      <c r="A54" t="s" s="2">
         <v>452</v>
       </c>
-      <c r="AO53" t="s" s="2">
-        <v>80</v>
-      </c>
-      <c r="AP53" t="s" s="2">
-        <v>80</v>
-      </c>
-      <c r="AQ53" t="s" s="2">
-        <v>453</v>
-      </c>
-    </row>
-    <row r="54">
-      <c r="A54" t="s" s="2">
-        <v>454</v>
-      </c>
       <c r="B54" t="s" s="2">
-        <v>454</v>
+        <v>452</v>
       </c>
       <c r="C54" s="2"/>
       <c r="D54" t="s" s="2">
@@ -8533,7 +8552,7 @@
         <v>93</v>
       </c>
       <c r="H54" t="s" s="2">
-        <v>94</v>
+        <v>80</v>
       </c>
       <c r="I54" t="s" s="2">
         <v>80</v>
@@ -8542,16 +8561,16 @@
         <v>94</v>
       </c>
       <c r="K54" t="s" s="2">
-        <v>315</v>
+        <v>147</v>
       </c>
       <c r="L54" t="s" s="2">
+        <v>453</v>
+      </c>
+      <c r="M54" t="s" s="2">
+        <v>454</v>
+      </c>
+      <c r="N54" t="s" s="2">
         <v>455</v>
-      </c>
-      <c r="M54" t="s" s="2">
-        <v>456</v>
-      </c>
-      <c r="N54" t="s" s="2">
-        <v>457</v>
       </c>
       <c r="O54" s="2"/>
       <c r="P54" t="s" s="2">
@@ -8577,13 +8596,13 @@
         <v>80</v>
       </c>
       <c r="X54" t="s" s="2">
-        <v>80</v>
+        <v>173</v>
       </c>
       <c r="Y54" t="s" s="2">
-        <v>80</v>
+        <v>456</v>
       </c>
       <c r="Z54" t="s" s="2">
-        <v>80</v>
+        <v>457</v>
       </c>
       <c r="AA54" t="s" s="2">
         <v>80</v>
@@ -8601,7 +8620,7 @@
         <v>80</v>
       </c>
       <c r="AF54" t="s" s="2">
-        <v>454</v>
+        <v>452</v>
       </c>
       <c r="AG54" t="s" s="2">
         <v>81</v>
@@ -8619,13 +8638,13 @@
         <v>80</v>
       </c>
       <c r="AL54" t="s" s="2">
-        <v>80</v>
+        <v>458</v>
       </c>
       <c r="AM54" t="s" s="2">
-        <v>458</v>
+        <v>374</v>
       </c>
       <c r="AN54" t="s" s="2">
-        <v>80</v>
+        <v>459</v>
       </c>
       <c r="AO54" t="s" s="2">
         <v>80</v>
@@ -8634,15 +8653,15 @@
         <v>80</v>
       </c>
       <c r="AQ54" t="s" s="2">
-        <v>80</v>
+        <v>460</v>
       </c>
     </row>
-    <row r="55" hidden="true">
+    <row r="55">
       <c r="A55" t="s" s="2">
-        <v>459</v>
+        <v>461</v>
       </c>
       <c r="B55" t="s" s="2">
-        <v>459</v>
+        <v>461</v>
       </c>
       <c r="C55" s="2"/>
       <c r="D55" t="s" s="2">
@@ -8656,24 +8675,26 @@
         <v>93</v>
       </c>
       <c r="H55" t="s" s="2">
-        <v>80</v>
+        <v>94</v>
       </c>
       <c r="I55" t="s" s="2">
         <v>80</v>
       </c>
       <c r="J55" t="s" s="2">
-        <v>80</v>
+        <v>94</v>
       </c>
       <c r="K55" t="s" s="2">
-        <v>107</v>
+        <v>322</v>
       </c>
       <c r="L55" t="s" s="2">
-        <v>108</v>
+        <v>462</v>
       </c>
       <c r="M55" t="s" s="2">
-        <v>109</v>
-      </c>
-      <c r="N55" s="2"/>
+        <v>463</v>
+      </c>
+      <c r="N55" t="s" s="2">
+        <v>464</v>
+      </c>
       <c r="O55" s="2"/>
       <c r="P55" t="s" s="2">
         <v>80</v>
@@ -8722,7 +8743,7 @@
         <v>80</v>
       </c>
       <c r="AF55" t="s" s="2">
-        <v>110</v>
+        <v>461</v>
       </c>
       <c r="AG55" t="s" s="2">
         <v>81</v>
@@ -8734,7 +8755,7 @@
         <v>80</v>
       </c>
       <c r="AJ55" t="s" s="2">
-        <v>80</v>
+        <v>105</v>
       </c>
       <c r="AK55" t="s" s="2">
         <v>80</v>
@@ -8743,7 +8764,7 @@
         <v>80</v>
       </c>
       <c r="AM55" t="s" s="2">
-        <v>111</v>
+        <v>465</v>
       </c>
       <c r="AN55" t="s" s="2">
         <v>80</v>
@@ -8760,21 +8781,21 @@
     </row>
     <row r="56" hidden="true">
       <c r="A56" t="s" s="2">
-        <v>460</v>
+        <v>466</v>
       </c>
       <c r="B56" t="s" s="2">
-        <v>460</v>
+        <v>466</v>
       </c>
       <c r="C56" s="2"/>
       <c r="D56" t="s" s="2">
-        <v>113</v>
+        <v>80</v>
       </c>
       <c r="E56" s="2"/>
       <c r="F56" t="s" s="2">
         <v>81</v>
       </c>
       <c r="G56" t="s" s="2">
-        <v>82</v>
+        <v>93</v>
       </c>
       <c r="H56" t="s" s="2">
         <v>80</v>
@@ -8786,17 +8807,15 @@
         <v>80</v>
       </c>
       <c r="K56" t="s" s="2">
-        <v>114</v>
+        <v>107</v>
       </c>
       <c r="L56" t="s" s="2">
-        <v>115</v>
+        <v>108</v>
       </c>
       <c r="M56" t="s" s="2">
-        <v>116</v>
-      </c>
-      <c r="N56" t="s" s="2">
-        <v>117</v>
-      </c>
+        <v>109</v>
+      </c>
+      <c r="N56" s="2"/>
       <c r="O56" s="2"/>
       <c r="P56" t="s" s="2">
         <v>80</v>
@@ -8845,19 +8864,19 @@
         <v>80</v>
       </c>
       <c r="AF56" t="s" s="2">
-        <v>121</v>
+        <v>110</v>
       </c>
       <c r="AG56" t="s" s="2">
         <v>81</v>
       </c>
       <c r="AH56" t="s" s="2">
-        <v>82</v>
+        <v>93</v>
       </c>
       <c r="AI56" t="s" s="2">
         <v>80</v>
       </c>
       <c r="AJ56" t="s" s="2">
-        <v>122</v>
+        <v>80</v>
       </c>
       <c r="AK56" t="s" s="2">
         <v>80</v>
@@ -8883,14 +8902,14 @@
     </row>
     <row r="57" hidden="true">
       <c r="A57" t="s" s="2">
-        <v>461</v>
+        <v>467</v>
       </c>
       <c r="B57" t="s" s="2">
-        <v>461</v>
+        <v>467</v>
       </c>
       <c r="C57" s="2"/>
       <c r="D57" t="s" s="2">
-        <v>325</v>
+        <v>113</v>
       </c>
       <c r="E57" s="2"/>
       <c r="F57" t="s" s="2">
@@ -8903,26 +8922,24 @@
         <v>80</v>
       </c>
       <c r="I57" t="s" s="2">
-        <v>94</v>
+        <v>80</v>
       </c>
       <c r="J57" t="s" s="2">
-        <v>94</v>
+        <v>80</v>
       </c>
       <c r="K57" t="s" s="2">
         <v>114</v>
       </c>
       <c r="L57" t="s" s="2">
-        <v>326</v>
+        <v>115</v>
       </c>
       <c r="M57" t="s" s="2">
-        <v>327</v>
+        <v>116</v>
       </c>
       <c r="N57" t="s" s="2">
         <v>117</v>
       </c>
-      <c r="O57" t="s" s="2">
-        <v>199</v>
-      </c>
+      <c r="O57" s="2"/>
       <c r="P57" t="s" s="2">
         <v>80</v>
       </c>
@@ -8970,7 +8987,7 @@
         <v>80</v>
       </c>
       <c r="AF57" t="s" s="2">
-        <v>328</v>
+        <v>121</v>
       </c>
       <c r="AG57" t="s" s="2">
         <v>81</v>
@@ -8991,7 +9008,7 @@
         <v>80</v>
       </c>
       <c r="AM57" t="s" s="2">
-        <v>192</v>
+        <v>111</v>
       </c>
       <c r="AN57" t="s" s="2">
         <v>80</v>
@@ -9006,16 +9023,16 @@
         <v>80</v>
       </c>
     </row>
-    <row r="58">
+    <row r="58" hidden="true">
       <c r="A58" t="s" s="2">
-        <v>462</v>
+        <v>468</v>
       </c>
       <c r="B58" t="s" s="2">
-        <v>462</v>
+        <v>468</v>
       </c>
       <c r="C58" s="2"/>
       <c r="D58" t="s" s="2">
-        <v>80</v>
+        <v>332</v>
       </c>
       <c r="E58" s="2"/>
       <c r="F58" t="s" s="2">
@@ -9025,25 +9042,29 @@
         <v>82</v>
       </c>
       <c r="H58" t="s" s="2">
+        <v>80</v>
+      </c>
+      <c r="I58" t="s" s="2">
         <v>94</v>
       </c>
-      <c r="I58" t="s" s="2">
-        <v>80</v>
-      </c>
       <c r="J58" t="s" s="2">
-        <v>80</v>
+        <v>94</v>
       </c>
       <c r="K58" t="s" s="2">
-        <v>463</v>
+        <v>114</v>
       </c>
       <c r="L58" t="s" s="2">
-        <v>464</v>
+        <v>333</v>
       </c>
       <c r="M58" t="s" s="2">
-        <v>465</v>
-      </c>
-      <c r="N58" s="2"/>
-      <c r="O58" s="2"/>
+        <v>334</v>
+      </c>
+      <c r="N58" t="s" s="2">
+        <v>117</v>
+      </c>
+      <c r="O58" t="s" s="2">
+        <v>206</v>
+      </c>
       <c r="P58" t="s" s="2">
         <v>80</v>
       </c>
@@ -9091,7 +9112,7 @@
         <v>80</v>
       </c>
       <c r="AF58" t="s" s="2">
-        <v>462</v>
+        <v>335</v>
       </c>
       <c r="AG58" t="s" s="2">
         <v>81</v>
@@ -9103,36 +9124,36 @@
         <v>80</v>
       </c>
       <c r="AJ58" t="s" s="2">
-        <v>105</v>
+        <v>122</v>
       </c>
       <c r="AK58" t="s" s="2">
-        <v>466</v>
+        <v>80</v>
       </c>
       <c r="AL58" t="s" s="2">
-        <v>467</v>
+        <v>80</v>
       </c>
       <c r="AM58" t="s" s="2">
-        <v>468</v>
+        <v>192</v>
       </c>
       <c r="AN58" t="s" s="2">
         <v>80</v>
       </c>
       <c r="AO58" t="s" s="2">
+        <v>80</v>
+      </c>
+      <c r="AP58" t="s" s="2">
+        <v>80</v>
+      </c>
+      <c r="AQ58" t="s" s="2">
+        <v>80</v>
+      </c>
+    </row>
+    <row r="59">
+      <c r="A59" t="s" s="2">
         <v>469</v>
       </c>
-      <c r="AP58" t="s" s="2">
-        <v>80</v>
-      </c>
-      <c r="AQ58" t="s" s="2">
-        <v>80</v>
-      </c>
-    </row>
-    <row r="59" hidden="true">
-      <c r="A59" t="s" s="2">
-        <v>470</v>
-      </c>
       <c r="B59" t="s" s="2">
-        <v>470</v>
+        <v>469</v>
       </c>
       <c r="C59" s="2"/>
       <c r="D59" t="s" s="2">
@@ -9146,7 +9167,7 @@
         <v>82</v>
       </c>
       <c r="H59" t="s" s="2">
-        <v>80</v>
+        <v>94</v>
       </c>
       <c r="I59" t="s" s="2">
         <v>80</v>
@@ -9155,7 +9176,7 @@
         <v>80</v>
       </c>
       <c r="K59" t="s" s="2">
-        <v>242</v>
+        <v>470</v>
       </c>
       <c r="L59" t="s" s="2">
         <v>471</v>
@@ -9163,9 +9184,7 @@
       <c r="M59" t="s" s="2">
         <v>472</v>
       </c>
-      <c r="N59" t="s" s="2">
-        <v>473</v>
-      </c>
+      <c r="N59" s="2"/>
       <c r="O59" s="2"/>
       <c r="P59" t="s" s="2">
         <v>80</v>
@@ -9190,13 +9209,13 @@
         <v>80</v>
       </c>
       <c r="X59" t="s" s="2">
-        <v>159</v>
+        <v>80</v>
       </c>
       <c r="Y59" t="s" s="2">
-        <v>474</v>
+        <v>80</v>
       </c>
       <c r="Z59" t="s" s="2">
-        <v>475</v>
+        <v>80</v>
       </c>
       <c r="AA59" t="s" s="2">
         <v>80</v>
@@ -9214,7 +9233,7 @@
         <v>80</v>
       </c>
       <c r="AF59" t="s" s="2">
-        <v>470</v>
+        <v>469</v>
       </c>
       <c r="AG59" t="s" s="2">
         <v>81</v>
@@ -9229,33 +9248,33 @@
         <v>105</v>
       </c>
       <c r="AK59" t="s" s="2">
-        <v>80</v>
+        <v>473</v>
       </c>
       <c r="AL59" t="s" s="2">
+        <v>474</v>
+      </c>
+      <c r="AM59" t="s" s="2">
+        <v>475</v>
+      </c>
+      <c r="AN59" t="s" s="2">
+        <v>80</v>
+      </c>
+      <c r="AO59" t="s" s="2">
         <v>476</v>
       </c>
-      <c r="AM59" t="s" s="2">
-        <v>477</v>
-      </c>
-      <c r="AN59" t="s" s="2">
-        <v>80</v>
-      </c>
-      <c r="AO59" t="s" s="2">
-        <v>80</v>
-      </c>
       <c r="AP59" t="s" s="2">
         <v>80</v>
       </c>
       <c r="AQ59" t="s" s="2">
-        <v>478</v>
+        <v>80</v>
       </c>
     </row>
     <row r="60" hidden="true">
       <c r="A60" t="s" s="2">
-        <v>479</v>
+        <v>477</v>
       </c>
       <c r="B60" t="s" s="2">
-        <v>479</v>
+        <v>477</v>
       </c>
       <c r="C60" s="2"/>
       <c r="D60" t="s" s="2">
@@ -9266,7 +9285,7 @@
         <v>81</v>
       </c>
       <c r="G60" t="s" s="2">
-        <v>93</v>
+        <v>82</v>
       </c>
       <c r="H60" t="s" s="2">
         <v>80</v>
@@ -9275,18 +9294,20 @@
         <v>80</v>
       </c>
       <c r="J60" t="s" s="2">
-        <v>94</v>
+        <v>80</v>
       </c>
       <c r="K60" t="s" s="2">
+        <v>249</v>
+      </c>
+      <c r="L60" t="s" s="2">
+        <v>478</v>
+      </c>
+      <c r="M60" t="s" s="2">
+        <v>479</v>
+      </c>
+      <c r="N60" t="s" s="2">
         <v>480</v>
       </c>
-      <c r="L60" t="s" s="2">
-        <v>481</v>
-      </c>
-      <c r="M60" t="s" s="2">
-        <v>482</v>
-      </c>
-      <c r="N60" s="2"/>
       <c r="O60" s="2"/>
       <c r="P60" t="s" s="2">
         <v>80</v>
@@ -9311,13 +9332,13 @@
         <v>80</v>
       </c>
       <c r="X60" t="s" s="2">
-        <v>80</v>
+        <v>159</v>
       </c>
       <c r="Y60" t="s" s="2">
-        <v>80</v>
+        <v>481</v>
       </c>
       <c r="Z60" t="s" s="2">
-        <v>80</v>
+        <v>482</v>
       </c>
       <c r="AA60" t="s" s="2">
         <v>80</v>
@@ -9335,13 +9356,13 @@
         <v>80</v>
       </c>
       <c r="AF60" t="s" s="2">
-        <v>479</v>
+        <v>477</v>
       </c>
       <c r="AG60" t="s" s="2">
         <v>81</v>
       </c>
       <c r="AH60" t="s" s="2">
-        <v>93</v>
+        <v>82</v>
       </c>
       <c r="AI60" t="s" s="2">
         <v>80</v>
@@ -9359,24 +9380,24 @@
         <v>484</v>
       </c>
       <c r="AN60" t="s" s="2">
+        <v>80</v>
+      </c>
+      <c r="AO60" t="s" s="2">
+        <v>80</v>
+      </c>
+      <c r="AP60" t="s" s="2">
+        <v>80</v>
+      </c>
+      <c r="AQ60" t="s" s="2">
         <v>485</v>
-      </c>
-      <c r="AO60" t="s" s="2">
-        <v>80</v>
-      </c>
-      <c r="AP60" t="s" s="2">
-        <v>80</v>
-      </c>
-      <c r="AQ60" t="s" s="2">
-        <v>486</v>
       </c>
     </row>
     <row r="61" hidden="true">
       <c r="A61" t="s" s="2">
-        <v>487</v>
+        <v>486</v>
       </c>
       <c r="B61" t="s" s="2">
-        <v>487</v>
+        <v>486</v>
       </c>
       <c r="C61" s="2"/>
       <c r="D61" t="s" s="2">
@@ -9396,10 +9417,10 @@
         <v>80</v>
       </c>
       <c r="J61" t="s" s="2">
-        <v>80</v>
+        <v>94</v>
       </c>
       <c r="K61" t="s" s="2">
-        <v>242</v>
+        <v>487</v>
       </c>
       <c r="L61" t="s" s="2">
         <v>488</v>
@@ -9432,13 +9453,13 @@
         <v>80</v>
       </c>
       <c r="X61" t="s" s="2">
-        <v>159</v>
+        <v>80</v>
       </c>
       <c r="Y61" t="s" s="2">
-        <v>490</v>
+        <v>80</v>
       </c>
       <c r="Z61" t="s" s="2">
-        <v>491</v>
+        <v>80</v>
       </c>
       <c r="AA61" t="s" s="2">
         <v>80</v>
@@ -9456,7 +9477,7 @@
         <v>80</v>
       </c>
       <c r="AF61" t="s" s="2">
-        <v>487</v>
+        <v>486</v>
       </c>
       <c r="AG61" t="s" s="2">
         <v>81</v>
@@ -9474,30 +9495,30 @@
         <v>80</v>
       </c>
       <c r="AL61" t="s" s="2">
+        <v>490</v>
+      </c>
+      <c r="AM61" t="s" s="2">
+        <v>491</v>
+      </c>
+      <c r="AN61" t="s" s="2">
         <v>492</v>
       </c>
-      <c r="AM61" t="s" s="2">
+      <c r="AO61" t="s" s="2">
+        <v>80</v>
+      </c>
+      <c r="AP61" t="s" s="2">
+        <v>80</v>
+      </c>
+      <c r="AQ61" t="s" s="2">
         <v>493</v>
-      </c>
-      <c r="AN61" t="s" s="2">
-        <v>494</v>
-      </c>
-      <c r="AO61" t="s" s="2">
-        <v>80</v>
-      </c>
-      <c r="AP61" t="s" s="2">
-        <v>80</v>
-      </c>
-      <c r="AQ61" t="s" s="2">
-        <v>495</v>
       </c>
     </row>
     <row r="62" hidden="true">
       <c r="A62" t="s" s="2">
-        <v>496</v>
+        <v>494</v>
       </c>
       <c r="B62" t="s" s="2">
-        <v>496</v>
+        <v>494</v>
       </c>
       <c r="C62" s="2"/>
       <c r="D62" t="s" s="2">
@@ -9520,20 +9541,16 @@
         <v>80</v>
       </c>
       <c r="K62" t="s" s="2">
-        <v>242</v>
+        <v>249</v>
       </c>
       <c r="L62" t="s" s="2">
-        <v>497</v>
+        <v>495</v>
       </c>
       <c r="M62" t="s" s="2">
-        <v>498</v>
-      </c>
-      <c r="N62" t="s" s="2">
-        <v>499</v>
-      </c>
-      <c r="O62" t="s" s="2">
-        <v>500</v>
-      </c>
+        <v>496</v>
+      </c>
+      <c r="N62" s="2"/>
+      <c r="O62" s="2"/>
       <c r="P62" t="s" s="2">
         <v>80</v>
       </c>
@@ -9560,10 +9577,10 @@
         <v>159</v>
       </c>
       <c r="Y62" t="s" s="2">
-        <v>501</v>
+        <v>497</v>
       </c>
       <c r="Z62" t="s" s="2">
-        <v>502</v>
+        <v>498</v>
       </c>
       <c r="AA62" t="s" s="2">
         <v>80</v>
@@ -9581,7 +9598,7 @@
         <v>80</v>
       </c>
       <c r="AF62" t="s" s="2">
-        <v>496</v>
+        <v>494</v>
       </c>
       <c r="AG62" t="s" s="2">
         <v>81</v>
@@ -9599,13 +9616,13 @@
         <v>80</v>
       </c>
       <c r="AL62" t="s" s="2">
-        <v>492</v>
+        <v>499</v>
       </c>
       <c r="AM62" t="s" s="2">
-        <v>493</v>
+        <v>500</v>
       </c>
       <c r="AN62" t="s" s="2">
-        <v>492</v>
+        <v>501</v>
       </c>
       <c r="AO62" t="s" s="2">
         <v>80</v>
@@ -9614,15 +9631,15 @@
         <v>80</v>
       </c>
       <c r="AQ62" t="s" s="2">
-        <v>503</v>
+        <v>502</v>
       </c>
     </row>
     <row r="63" hidden="true">
       <c r="A63" t="s" s="2">
-        <v>504</v>
+        <v>503</v>
       </c>
       <c r="B63" t="s" s="2">
-        <v>504</v>
+        <v>503</v>
       </c>
       <c r="C63" s="2"/>
       <c r="D63" t="s" s="2">
@@ -9645,16 +9662,20 @@
         <v>80</v>
       </c>
       <c r="K63" t="s" s="2">
+        <v>249</v>
+      </c>
+      <c r="L63" t="s" s="2">
+        <v>504</v>
+      </c>
+      <c r="M63" t="s" s="2">
         <v>505</v>
       </c>
-      <c r="L63" t="s" s="2">
+      <c r="N63" t="s" s="2">
         <v>506</v>
       </c>
-      <c r="M63" t="s" s="2">
+      <c r="O63" t="s" s="2">
         <v>507</v>
       </c>
-      <c r="N63" s="2"/>
-      <c r="O63" s="2"/>
       <c r="P63" t="s" s="2">
         <v>80</v>
       </c>
@@ -9678,13 +9699,13 @@
         <v>80</v>
       </c>
       <c r="X63" t="s" s="2">
-        <v>80</v>
+        <v>159</v>
       </c>
       <c r="Y63" t="s" s="2">
-        <v>80</v>
+        <v>508</v>
       </c>
       <c r="Z63" t="s" s="2">
-        <v>80</v>
+        <v>509</v>
       </c>
       <c r="AA63" t="s" s="2">
         <v>80</v>
@@ -9702,7 +9723,7 @@
         <v>80</v>
       </c>
       <c r="AF63" t="s" s="2">
-        <v>504</v>
+        <v>503</v>
       </c>
       <c r="AG63" t="s" s="2">
         <v>81</v>
@@ -9720,13 +9741,13 @@
         <v>80</v>
       </c>
       <c r="AL63" t="s" s="2">
-        <v>271</v>
+        <v>499</v>
       </c>
       <c r="AM63" t="s" s="2">
-        <v>272</v>
+        <v>500</v>
       </c>
       <c r="AN63" t="s" s="2">
-        <v>273</v>
+        <v>499</v>
       </c>
       <c r="AO63" t="s" s="2">
         <v>80</v>
@@ -9735,15 +9756,15 @@
         <v>80</v>
       </c>
       <c r="AQ63" t="s" s="2">
-        <v>508</v>
+        <v>510</v>
       </c>
     </row>
     <row r="64" hidden="true">
       <c r="A64" t="s" s="2">
-        <v>509</v>
+        <v>511</v>
       </c>
       <c r="B64" t="s" s="2">
-        <v>509</v>
+        <v>511</v>
       </c>
       <c r="C64" s="2"/>
       <c r="D64" t="s" s="2">
@@ -9754,7 +9775,7 @@
         <v>81</v>
       </c>
       <c r="G64" t="s" s="2">
-        <v>82</v>
+        <v>93</v>
       </c>
       <c r="H64" t="s" s="2">
         <v>80</v>
@@ -9766,17 +9787,15 @@
         <v>80</v>
       </c>
       <c r="K64" t="s" s="2">
-        <v>510</v>
+        <v>512</v>
       </c>
       <c r="L64" t="s" s="2">
-        <v>511</v>
+        <v>513</v>
       </c>
       <c r="M64" t="s" s="2">
-        <v>512</v>
-      </c>
-      <c r="N64" t="s" s="2">
-        <v>513</v>
-      </c>
+        <v>514</v>
+      </c>
+      <c r="N64" s="2"/>
       <c r="O64" s="2"/>
       <c r="P64" t="s" s="2">
         <v>80</v>
@@ -9825,13 +9844,13 @@
         <v>80</v>
       </c>
       <c r="AF64" t="s" s="2">
-        <v>509</v>
+        <v>511</v>
       </c>
       <c r="AG64" t="s" s="2">
         <v>81</v>
       </c>
       <c r="AH64" t="s" s="2">
-        <v>82</v>
+        <v>93</v>
       </c>
       <c r="AI64" t="s" s="2">
         <v>80</v>
@@ -9843,26 +9862,149 @@
         <v>80</v>
       </c>
       <c r="AL64" t="s" s="2">
-        <v>514</v>
+        <v>278</v>
       </c>
       <c r="AM64" t="s" s="2">
+        <v>279</v>
+      </c>
+      <c r="AN64" t="s" s="2">
+        <v>280</v>
+      </c>
+      <c r="AO64" t="s" s="2">
+        <v>80</v>
+      </c>
+      <c r="AP64" t="s" s="2">
+        <v>80</v>
+      </c>
+      <c r="AQ64" t="s" s="2">
         <v>515</v>
       </c>
-      <c r="AN64" t="s" s="2">
+    </row>
+    <row r="65" hidden="true">
+      <c r="A65" t="s" s="2">
         <v>516</v>
       </c>
-      <c r="AO64" t="s" s="2">
-        <v>80</v>
-      </c>
-      <c r="AP64" t="s" s="2">
-        <v>80</v>
-      </c>
-      <c r="AQ64" t="s" s="2">
+      <c r="B65" t="s" s="2">
+        <v>516</v>
+      </c>
+      <c r="C65" s="2"/>
+      <c r="D65" t="s" s="2">
+        <v>80</v>
+      </c>
+      <c r="E65" s="2"/>
+      <c r="F65" t="s" s="2">
+        <v>81</v>
+      </c>
+      <c r="G65" t="s" s="2">
+        <v>82</v>
+      </c>
+      <c r="H65" t="s" s="2">
+        <v>80</v>
+      </c>
+      <c r="I65" t="s" s="2">
+        <v>80</v>
+      </c>
+      <c r="J65" t="s" s="2">
+        <v>80</v>
+      </c>
+      <c r="K65" t="s" s="2">
         <v>517</v>
+      </c>
+      <c r="L65" t="s" s="2">
+        <v>518</v>
+      </c>
+      <c r="M65" t="s" s="2">
+        <v>519</v>
+      </c>
+      <c r="N65" t="s" s="2">
+        <v>520</v>
+      </c>
+      <c r="O65" s="2"/>
+      <c r="P65" t="s" s="2">
+        <v>80</v>
+      </c>
+      <c r="Q65" s="2"/>
+      <c r="R65" t="s" s="2">
+        <v>80</v>
+      </c>
+      <c r="S65" t="s" s="2">
+        <v>80</v>
+      </c>
+      <c r="T65" t="s" s="2">
+        <v>80</v>
+      </c>
+      <c r="U65" t="s" s="2">
+        <v>80</v>
+      </c>
+      <c r="V65" t="s" s="2">
+        <v>80</v>
+      </c>
+      <c r="W65" t="s" s="2">
+        <v>80</v>
+      </c>
+      <c r="X65" t="s" s="2">
+        <v>80</v>
+      </c>
+      <c r="Y65" t="s" s="2">
+        <v>80</v>
+      </c>
+      <c r="Z65" t="s" s="2">
+        <v>80</v>
+      </c>
+      <c r="AA65" t="s" s="2">
+        <v>80</v>
+      </c>
+      <c r="AB65" t="s" s="2">
+        <v>80</v>
+      </c>
+      <c r="AC65" t="s" s="2">
+        <v>80</v>
+      </c>
+      <c r="AD65" t="s" s="2">
+        <v>80</v>
+      </c>
+      <c r="AE65" t="s" s="2">
+        <v>80</v>
+      </c>
+      <c r="AF65" t="s" s="2">
+        <v>516</v>
+      </c>
+      <c r="AG65" t="s" s="2">
+        <v>81</v>
+      </c>
+      <c r="AH65" t="s" s="2">
+        <v>82</v>
+      </c>
+      <c r="AI65" t="s" s="2">
+        <v>80</v>
+      </c>
+      <c r="AJ65" t="s" s="2">
+        <v>105</v>
+      </c>
+      <c r="AK65" t="s" s="2">
+        <v>80</v>
+      </c>
+      <c r="AL65" t="s" s="2">
+        <v>521</v>
+      </c>
+      <c r="AM65" t="s" s="2">
+        <v>522</v>
+      </c>
+      <c r="AN65" t="s" s="2">
+        <v>523</v>
+      </c>
+      <c r="AO65" t="s" s="2">
+        <v>80</v>
+      </c>
+      <c r="AP65" t="s" s="2">
+        <v>80</v>
+      </c>
+      <c r="AQ65" t="s" s="2">
+        <v>524</v>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:AQ64">
+  <autoFilter ref="A1:AQ65">
     <filterColumn colId="7">
       <customFilters>
         <customFilter operator="notEqual" val=" "/>
@@ -9872,7 +10014,7 @@
       <filters blank="true"/>
     </filterColumn>
   </autoFilter>
-  <conditionalFormatting sqref="A2:AI63">
+  <conditionalFormatting sqref="A2:AI64">
     <cfRule type="expression" dxfId="0" priority="1">
       <formula>$G2&lt;&gt;"Y"</formula>
     </cfRule>

</xml_diff>